<commit_message>
fmkadc working alsmost finished
</commit_message>
<xml_diff>
--- a/Doc/ConfigPrj/ExcelCfg/STM32G474RE/STM32G474RE_HwCfg.xlsx
+++ b/Doc/ConfigPrj/ExcelCfg/STM32G474RE/STM32G474RE_HwCfg.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\Software\STM32\f_designHRTIM\Doc\ConfigPrj\ExcelCfg\STM32G474RE\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\Software\STM32\Gamma_fCreateCfg\Doc\ConfigPrj\ExcelCfg\STM32G474RE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EA82B7E-77D6-4C6B-95E5-686F4DB99418}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44571CCE-BEEE-4655-BC7D-C952B91BC2FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{2AF09063-600F-437A-B138-F66136E922A5}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{2AF09063-600F-437A-B138-F66136E922A5}"/>
   </bookViews>
   <sheets>
     <sheet name="General_Info" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1058" uniqueCount="481">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1067" uniqueCount="487">
   <si>
     <t>Colonne1</t>
   </si>
@@ -1488,6 +1488,24 @@
   </si>
   <si>
     <t>ADC_CHANNEL_18</t>
+  </si>
+  <si>
+    <t>Channel spec</t>
+  </si>
+  <si>
+    <t>VBAT</t>
+  </si>
+  <si>
+    <t>0x00000000</t>
+  </si>
+  <si>
+    <t>Enable</t>
+  </si>
+  <si>
+    <t>TRUE</t>
+  </si>
+  <si>
+    <t>FALSE</t>
   </si>
 </sst>
 </file>
@@ -4164,13 +4182,14 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{A27CADD5-26F4-4DF6-9D41-CEE02A85C4E9}" name="GI_ADC" displayName="GI_ADC" ref="V40:Y45" totalsRowShown="0">
-  <autoFilter ref="V40:Y45" xr:uid="{A27CADD5-26F4-4DF6-9D41-CEE02A85C4E9}"/>
-  <tableColumns count="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{A27CADD5-26F4-4DF6-9D41-CEE02A85C4E9}" name="GI_ADC" displayName="GI_ADC" ref="V40:Z45" totalsRowShown="0">
+  <autoFilter ref="V40:Z45" xr:uid="{A27CADD5-26F4-4DF6-9D41-CEE02A85C4E9}"/>
+  <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{46462DEE-B3A7-45AD-A2F8-63AC8C3C0154}" name="ADC_Name"/>
     <tableColumn id="2" xr3:uid="{20DF5352-4B39-416D-A6E4-D94E56AED1C9}" name="number of channel"/>
     <tableColumn id="3" xr3:uid="{9F9316C2-2066-47BF-B84E-436D4C41B07C}" name="IRQN assoiated"/>
     <tableColumn id="4" xr3:uid="{CC116C4D-98B0-46BC-A882-0B90828FFD68}" name="Clock Associated"/>
+    <tableColumn id="5" xr3:uid="{06173FC1-6C9B-4FF4-AB3F-A7854D314A0A}" name="Channel spec"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4378,13 +4397,14 @@
 </file>
 
 <file path=xl/tables/table29.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="24" xr:uid="{A4F27ADC-56A6-479B-93EF-D6AA72368D72}" name="FMKCDA_CalibrationOthers" displayName="FMKCDA_CalibrationOthers" ref="I3:L5" totalsRowShown="0">
-  <autoFilter ref="I3:L5" xr:uid="{A4F27ADC-56A6-479B-93EF-D6AA72368D72}"/>
-  <tableColumns count="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="24" xr:uid="{A4F27ADC-56A6-479B-93EF-D6AA72368D72}" name="FMKCDA_CalibrationOthers" displayName="FMKCDA_CalibrationOthers" ref="I3:M6" totalsRowShown="0">
+  <autoFilter ref="I3:M6" xr:uid="{A4F27ADC-56A6-479B-93EF-D6AA72368D72}"/>
+  <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{74AD6856-B046-40F9-89E8-C5AC0EB4C661}" name="calibration temperature "/>
     <tableColumn id="2" xr3:uid="{D58B2B24-74EC-4445-9DDA-83A119877B67}" name="address in hexacecimal"/>
     <tableColumn id="3" xr3:uid="{0793AAF2-321B-4695-AEBB-122FAB9D49F7}" name="Adc Vref"/>
     <tableColumn id="4" xr3:uid="{F1198D75-5BAD-4CA5-814F-DDA2BB66E5F2}" name="Channel Vref"/>
+    <tableColumn id="5" xr3:uid="{6C202CA4-44FC-4E46-A4B5-AF7389AC3A4D}" name="Enable"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4402,8 +4422,8 @@
 </file>
 
 <file path=xl/tables/table30.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="25" xr:uid="{99B4503A-67B2-48AD-BE25-2B3425F892A9}" name="FMKCDA_VoltageRef" displayName="FMKCDA_VoltageRef" ref="S3:V8" totalsRowShown="0">
-  <autoFilter ref="S3:V8" xr:uid="{99B4503A-67B2-48AD-BE25-2B3425F892A9}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="25" xr:uid="{99B4503A-67B2-48AD-BE25-2B3425F892A9}" name="FMKCDA_VoltageRef" displayName="FMKCDA_VoltageRef" ref="T17:W22" totalsRowShown="0">
+  <autoFilter ref="T17:W22" xr:uid="{99B4503A-67B2-48AD-BE25-2B3425F892A9}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{0BCC2BC4-7FF0-4C14-809D-9D95A3225151}" name="Vref Calib"/>
     <tableColumn id="2" xr3:uid="{0E78A6D4-DF9E-4966-A80E-64FE5BD9F1E2}" name="address  hexacecimal"/>
@@ -4535,8 +4555,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{13E9277E-229F-41F0-9B99-7D1A0B71D1B3}" name="Tableau16" displayName="Tableau16" ref="AF40:AF43" totalsRowShown="0">
-  <autoFilter ref="AF40:AF43" xr:uid="{13E9277E-229F-41F0-9B99-7D1A0B71D1B3}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{13E9277E-229F-41F0-9B99-7D1A0B71D1B3}" name="Tableau16" displayName="Tableau16" ref="AG40:AG43" totalsRowShown="0">
+  <autoFilter ref="AG40:AG43" xr:uid="{13E9277E-229F-41F0-9B99-7D1A0B71D1B3}"/>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{84137467-8FB1-43EA-9F20-573D7FE9FADD}" name="_NVIC_Piority_Choice"/>
   </tableColumns>
@@ -4881,7 +4901,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{871E2D6D-43F7-44B1-8255-ECFDDA33AA9C}">
-  <dimension ref="A17:AF119"/>
+  <dimension ref="A17:AG119"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23.6640625" customWidth="1"/>
@@ -4906,6 +4926,7 @@
     <col min="22" max="22" width="19.109375" customWidth="1"/>
     <col min="23" max="23" width="18.77734375" customWidth="1"/>
     <col min="24" max="24" width="29.21875" customWidth="1"/>
+    <col min="26" max="26" width="17.44140625" customWidth="1"/>
     <col min="28" max="28" width="24" customWidth="1"/>
     <col min="31" max="31" width="17.77734375" customWidth="1"/>
   </cols>
@@ -5431,7 +5452,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="33" spans="4:32" x14ac:dyDescent="0.3">
+    <row r="33" spans="4:33" x14ac:dyDescent="0.3">
       <c r="D33" t="s">
         <v>237</v>
       </c>
@@ -5454,7 +5475,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="34" spans="4:32" x14ac:dyDescent="0.3">
+    <row r="34" spans="4:33" x14ac:dyDescent="0.3">
       <c r="D34" t="s">
         <v>238</v>
       </c>
@@ -5477,7 +5498,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="35" spans="4:32" x14ac:dyDescent="0.3">
+    <row r="35" spans="4:33" x14ac:dyDescent="0.3">
       <c r="D35" t="s">
         <v>229</v>
       </c>
@@ -5500,7 +5521,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="36" spans="4:32" x14ac:dyDescent="0.3">
+    <row r="36" spans="4:33" x14ac:dyDescent="0.3">
       <c r="D36" t="s">
         <v>228</v>
       </c>
@@ -5529,7 +5550,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="37" spans="4:32" x14ac:dyDescent="0.3">
+    <row r="37" spans="4:33" x14ac:dyDescent="0.3">
       <c r="D37" t="s">
         <v>239</v>
       </c>
@@ -5558,7 +5579,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="38" spans="4:32" x14ac:dyDescent="0.3">
+    <row r="38" spans="4:33" x14ac:dyDescent="0.3">
       <c r="D38" t="s">
         <v>240</v>
       </c>
@@ -5581,7 +5602,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="39" spans="4:32" x14ac:dyDescent="0.3">
+    <row r="39" spans="4:33" x14ac:dyDescent="0.3">
       <c r="D39" t="s">
         <v>215</v>
       </c>
@@ -5604,7 +5625,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="40" spans="4:32" x14ac:dyDescent="0.3">
+    <row r="40" spans="4:33" x14ac:dyDescent="0.3">
       <c r="D40" t="s">
         <v>241</v>
       </c>
@@ -5638,11 +5659,14 @@
       <c r="Y40" t="s">
         <v>276</v>
       </c>
-      <c r="AF40" t="s">
+      <c r="Z40" t="s">
+        <v>481</v>
+      </c>
+      <c r="AG40" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="41" spans="4:32" x14ac:dyDescent="0.3">
+    <row r="41" spans="4:33" x14ac:dyDescent="0.3">
       <c r="D41" t="s">
         <v>242</v>
       </c>
@@ -5670,11 +5694,11 @@
       <c r="Y41" t="s">
         <v>237</v>
       </c>
-      <c r="AF41" t="s">
+      <c r="AG41" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="42" spans="4:32" x14ac:dyDescent="0.3">
+    <row r="42" spans="4:33" x14ac:dyDescent="0.3">
       <c r="D42" t="s">
         <v>227</v>
       </c>
@@ -5702,11 +5726,11 @@
       <c r="Y42" t="s">
         <v>237</v>
       </c>
-      <c r="AF42" t="s">
+      <c r="AG42" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="43" spans="4:32" x14ac:dyDescent="0.3">
+    <row r="43" spans="4:33" x14ac:dyDescent="0.3">
       <c r="D43" t="s">
         <v>72</v>
       </c>
@@ -5734,11 +5758,11 @@
       <c r="Y43" t="s">
         <v>238</v>
       </c>
-      <c r="AF43" t="s">
+      <c r="AG43" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="44" spans="4:32" x14ac:dyDescent="0.3">
+    <row r="44" spans="4:33" x14ac:dyDescent="0.3">
       <c r="D44" t="s">
         <v>226</v>
       </c>
@@ -5767,7 +5791,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="45" spans="4:32" x14ac:dyDescent="0.3">
+    <row r="45" spans="4:33" x14ac:dyDescent="0.3">
       <c r="D45" t="s">
         <v>243</v>
       </c>
@@ -5796,7 +5820,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="46" spans="4:32" x14ac:dyDescent="0.3">
+    <row r="46" spans="4:33" x14ac:dyDescent="0.3">
       <c r="D46" t="s">
         <v>225</v>
       </c>
@@ -5816,7 +5840,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="47" spans="4:32" x14ac:dyDescent="0.3">
+    <row r="47" spans="4:33" x14ac:dyDescent="0.3">
       <c r="D47" t="s">
         <v>224</v>
       </c>
@@ -5836,7 +5860,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="48" spans="4:32" x14ac:dyDescent="0.3">
+    <row r="48" spans="4:33" x14ac:dyDescent="0.3">
       <c r="D48" t="s">
         <v>244</v>
       </c>
@@ -6707,7 +6731,7 @@
   <phoneticPr fontId="1" type="noConversion"/>
   <dataValidations count="4">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I18:I119" xr:uid="{AAB57854-EE21-4648-A1CB-0F7D2F2AF990}">
-      <formula1>$AF$41:$AF$43</formula1>
+      <formula1>$AG$41:$AG$43</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N19:N30" xr:uid="{FCBABE9C-10FE-40A4-8AA4-1BAED7C63E26}">
       <formula1>$AF$47:$AF$49</formula1>
@@ -6973,6 +6997,7 @@
     <col min="31" max="31" width="17.6640625" customWidth="1"/>
     <col min="38" max="38" width="17.21875" customWidth="1"/>
     <col min="40" max="40" width="19.44140625" customWidth="1"/>
+    <col min="53" max="53" width="40.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:28" x14ac:dyDescent="0.3">
@@ -8193,7 +8218,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0962FBCC-E1F3-44E3-92A8-D1FF17927B08}">
-  <dimension ref="E2:V12"/>
+  <dimension ref="E2:W22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="5" max="5" width="23.44140625" customWidth="1"/>
@@ -8209,7 +8234,7 @@
     <col min="22" max="22" width="18.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="5:22" ht="25.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="5:17" ht="25.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="I2" s="3" t="s">
         <v>117</v>
       </c>
@@ -8217,7 +8242,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="3" spans="5:22" x14ac:dyDescent="0.3">
+    <row r="3" spans="5:17" x14ac:dyDescent="0.3">
       <c r="I3" t="s">
         <v>114</v>
       </c>
@@ -8230,123 +8255,75 @@
       <c r="L3" t="s">
         <v>119</v>
       </c>
-      <c r="S3" t="s">
-        <v>116</v>
-      </c>
-      <c r="T3" t="s">
-        <v>121</v>
-      </c>
-      <c r="U3" t="s">
-        <v>118</v>
-      </c>
-      <c r="V3" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="4" spans="5:22" x14ac:dyDescent="0.3">
+      <c r="M3" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="4" spans="5:17" x14ac:dyDescent="0.3">
       <c r="I4" t="s">
-        <v>113</v>
+        <v>482</v>
       </c>
       <c r="J4" t="s">
-        <v>266</v>
+        <v>483</v>
       </c>
       <c r="K4" t="s">
         <v>16</v>
       </c>
       <c r="L4" t="s">
+        <v>111</v>
+      </c>
+      <c r="M4" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="5" spans="5:17" x14ac:dyDescent="0.3">
+      <c r="I5" t="s">
+        <v>113</v>
+      </c>
+      <c r="J5" t="s">
+        <v>266</v>
+      </c>
+      <c r="K5" t="s">
+        <v>16</v>
+      </c>
+      <c r="L5" t="s">
         <v>110</v>
       </c>
-      <c r="S4" t="s">
-        <v>419</v>
-      </c>
-      <c r="T4" t="s">
-        <v>268</v>
-      </c>
-      <c r="U4" t="s">
-        <v>16</v>
-      </c>
-      <c r="V4" t="s">
-        <v>480</v>
-      </c>
-    </row>
-    <row r="5" spans="5:22" x14ac:dyDescent="0.3">
-      <c r="I5" t="s">
+      <c r="M5" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="6" spans="5:17" x14ac:dyDescent="0.3">
+      <c r="I6" t="s">
         <v>265</v>
       </c>
-      <c r="J5" t="s">
+      <c r="J6" t="s">
         <v>267</v>
       </c>
-      <c r="K5" t="s">
+      <c r="K6" t="s">
         <v>264</v>
       </c>
-      <c r="L5" t="s">
+      <c r="L6" t="s">
         <v>98</v>
       </c>
-      <c r="S5" t="s">
-        <v>420</v>
-      </c>
-      <c r="T5" t="s">
-        <v>268</v>
-      </c>
-      <c r="U5" t="s">
-        <v>16</v>
-      </c>
-      <c r="V5" t="s">
-        <v>480</v>
-      </c>
-    </row>
-    <row r="6" spans="5:22" x14ac:dyDescent="0.3">
-      <c r="S6" t="s">
-        <v>421</v>
-      </c>
-      <c r="T6" t="s">
-        <v>268</v>
-      </c>
-      <c r="U6" t="s">
-        <v>262</v>
-      </c>
-      <c r="V6" t="s">
-        <v>480</v>
-      </c>
-    </row>
-    <row r="7" spans="5:22" x14ac:dyDescent="0.3">
+      <c r="M6" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="7" spans="5:17" x14ac:dyDescent="0.3">
       <c r="E7" t="s">
         <v>360</v>
       </c>
-      <c r="S7" t="s">
-        <v>422</v>
-      </c>
-      <c r="T7" t="s">
-        <v>268</v>
-      </c>
-      <c r="U7" t="s">
-        <v>263</v>
-      </c>
-      <c r="V7" t="s">
-        <v>480</v>
-      </c>
-    </row>
-    <row r="8" spans="5:22" x14ac:dyDescent="0.3">
+    </row>
+    <row r="8" spans="5:17" x14ac:dyDescent="0.3">
       <c r="E8" t="s">
         <v>353</v>
       </c>
       <c r="F8" t="s">
         <v>395</v>
       </c>
-      <c r="S8" t="s">
-        <v>423</v>
-      </c>
-      <c r="T8" t="s">
-        <v>268</v>
-      </c>
-      <c r="U8" t="s">
-        <v>264</v>
-      </c>
-      <c r="V8" t="s">
-        <v>480</v>
-      </c>
-    </row>
-    <row r="9" spans="5:22" x14ac:dyDescent="0.3">
+    </row>
+    <row r="9" spans="5:17" x14ac:dyDescent="0.3">
       <c r="E9" t="s">
         <v>368</v>
       </c>
@@ -8354,7 +8331,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="10" spans="5:22" x14ac:dyDescent="0.3">
+    <row r="10" spans="5:17" x14ac:dyDescent="0.3">
       <c r="E10" t="s">
         <v>369</v>
       </c>
@@ -8362,7 +8339,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="11" spans="5:22" x14ac:dyDescent="0.3">
+    <row r="11" spans="5:17" x14ac:dyDescent="0.3">
       <c r="E11" t="s">
         <v>370</v>
       </c>
@@ -8370,12 +8347,96 @@
         <v>398</v>
       </c>
     </row>
-    <row r="12" spans="5:22" x14ac:dyDescent="0.3">
+    <row r="12" spans="5:17" x14ac:dyDescent="0.3">
       <c r="E12" t="s">
         <v>371</v>
       </c>
       <c r="F12" t="s">
         <v>399</v>
+      </c>
+    </row>
+    <row r="17" spans="20:23" x14ac:dyDescent="0.3">
+      <c r="T17" t="s">
+        <v>116</v>
+      </c>
+      <c r="U17" t="s">
+        <v>121</v>
+      </c>
+      <c r="V17" t="s">
+        <v>118</v>
+      </c>
+      <c r="W17" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="18" spans="20:23" x14ac:dyDescent="0.3">
+      <c r="T18" t="s">
+        <v>419</v>
+      </c>
+      <c r="U18" t="s">
+        <v>268</v>
+      </c>
+      <c r="V18" t="s">
+        <v>16</v>
+      </c>
+      <c r="W18" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="19" spans="20:23" x14ac:dyDescent="0.3">
+      <c r="T19" t="s">
+        <v>420</v>
+      </c>
+      <c r="U19" t="s">
+        <v>268</v>
+      </c>
+      <c r="V19" t="s">
+        <v>16</v>
+      </c>
+      <c r="W19" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="20" spans="20:23" x14ac:dyDescent="0.3">
+      <c r="T20" t="s">
+        <v>421</v>
+      </c>
+      <c r="U20" t="s">
+        <v>268</v>
+      </c>
+      <c r="V20" t="s">
+        <v>262</v>
+      </c>
+      <c r="W20" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="21" spans="20:23" x14ac:dyDescent="0.3">
+      <c r="T21" t="s">
+        <v>422</v>
+      </c>
+      <c r="U21" t="s">
+        <v>268</v>
+      </c>
+      <c r="V21" t="s">
+        <v>263</v>
+      </c>
+      <c r="W21" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="22" spans="20:23" x14ac:dyDescent="0.3">
+      <c r="T22" t="s">
+        <v>423</v>
+      </c>
+      <c r="U22" t="s">
+        <v>268</v>
+      </c>
+      <c r="V22" t="s">
+        <v>264</v>
+      </c>
+      <c r="W22" t="s">
+        <v>480</v>
       </c>
     </row>
   </sheetData>
@@ -8393,13 +8454,13 @@
           <x14:formula1>
             <xm:f>General_Info!$V$41:$V$45</xm:f>
           </x14:formula1>
-          <xm:sqref>K4:K5 U4:U8</xm:sqref>
+          <xm:sqref>K4:K6 V18:V22</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{7AB0981D-B484-49AA-81E2-46EA728857EF}">
           <x14:formula1>
             <xm:f>FMK_IO!$BA$30:$BA$47</xm:f>
           </x14:formula1>
-          <xm:sqref>L4:L5</xm:sqref>
+          <xm:sqref>L4:L6</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>

<commit_message>
All framework working with adc/srl/ log perfet
</commit_message>
<xml_diff>
--- a/Doc/ConfigPrj/ExcelCfg/STM32G474RE/STM32G474RE_HwCfg.xlsx
+++ b/Doc/ConfigPrj/ExcelCfg/STM32G474RE/STM32G474RE_HwCfg.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\Software\STM32\Gamma_fCreateCfg\Doc\ConfigPrj\ExcelCfg\STM32G474RE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44571CCE-BEEE-4655-BC7D-C952B91BC2FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2BD330D-240E-41F1-9514-7F79FA8EA4DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{2AF09063-600F-437A-B138-F66136E922A5}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="7" xr2:uid="{2AF09063-600F-437A-B138-F66136E922A5}"/>
   </bookViews>
   <sheets>
     <sheet name="General_Info" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1067" uniqueCount="487">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1064" uniqueCount="495">
   <si>
     <t>Colonne1</t>
   </si>
@@ -1076,18 +1076,9 @@
     <t>CHANNEL_7</t>
   </si>
   <si>
-    <t>SERIAL CONFIGURATION</t>
-  </si>
-  <si>
     <t>GPIO_AF7_USART2</t>
   </si>
   <si>
-    <t>GPIO_AF5_UART4</t>
-  </si>
-  <si>
-    <t>UART/USART REF</t>
-  </si>
-  <si>
     <t>TIM1_BRK_TIM15_IRQHandler</t>
   </si>
   <si>
@@ -1484,9 +1475,6 @@
     <t>EXTI3_IRQN</t>
   </si>
   <si>
-    <t>EXTI4_IRQN</t>
-  </si>
-  <si>
     <t>ADC_CHANNEL_18</t>
   </si>
   <si>
@@ -1506,6 +1494,42 @@
   </si>
   <si>
     <t>FALSE</t>
+  </si>
+  <si>
+    <t>Instance</t>
+  </si>
+  <si>
+    <t>FDCAN1</t>
+  </si>
+  <si>
+    <t>RxBuffer Size</t>
+  </si>
+  <si>
+    <t>Tx buffer Size</t>
+  </si>
+  <si>
+    <t>FDCAN2</t>
+  </si>
+  <si>
+    <t>FDCAN3</t>
+  </si>
+  <si>
+    <t>RCC Clock</t>
+  </si>
+  <si>
+    <t>GPIO_AF9_FDCAN2</t>
+  </si>
+  <si>
+    <t>USART3_RX</t>
+  </si>
+  <si>
+    <t>USART3_TX</t>
+  </si>
+  <si>
+    <t>voir dans cubeMx associé enable register DMA</t>
+  </si>
+  <si>
+    <t>GPIO_AF11_FDCAN3</t>
   </si>
 </sst>
 </file>
@@ -4219,8 +4243,8 @@
 </file>
 
 <file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{098A48DC-88A9-4122-ADE1-86E0F3796141}" name="FMKIO_OutputDig" displayName="FMKIO_OutputDig" ref="AA7:AB17" totalsRowShown="0">
-  <autoFilter ref="AA7:AB17" xr:uid="{098A48DC-88A9-4122-ADE1-86E0F3796141}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{098A48DC-88A9-4122-ADE1-86E0F3796141}" name="FMKIO_OutputDig" displayName="FMKIO_OutputDig" ref="AA7:AB16" totalsRowShown="0">
+  <autoFilter ref="AA7:AB16" xr:uid="{098A48DC-88A9-4122-ADE1-86E0F3796141}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{395BD36A-0840-48CF-8D8D-56878E366FC5}" name="GPIO_name"/>
     <tableColumn id="2" xr3:uid="{34DF2CF3-8826-4F9E-A09D-280EE0FEFFBB}" name="Pin_name"/>
@@ -4244,8 +4268,8 @@
 </file>
 
 <file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{0918A5C3-EE53-4DBF-8C0C-2251FB41871E}" name="FMKIO_InputEvnt" displayName="FMKIO_InputEvnt" ref="W6:Y9" totalsRowShown="0">
-  <autoFilter ref="W6:Y9" xr:uid="{0918A5C3-EE53-4DBF-8C0C-2251FB41871E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{0918A5C3-EE53-4DBF-8C0C-2251FB41871E}" name="FMKIO_InputEvnt" displayName="FMKIO_InputEvnt" ref="W6:Y8" totalsRowShown="0">
+  <autoFilter ref="W6:Y8" xr:uid="{0918A5C3-EE53-4DBF-8C0C-2251FB41871E}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{5C8A98A4-9028-4F61-A263-67D85D1BFF84}" name="GPIO_name"/>
     <tableColumn id="2" xr3:uid="{D3F2DFB4-9CF8-4086-ABAA-63BD13D3A4C5}" name="Pin_name"/>
@@ -4340,23 +4364,8 @@
 </file>
 
 <file path=xl/tables/table24.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="30" xr:uid="{978057A4-13F6-44F3-B65B-2C409866E1DE}" name="FMKIO_SerialCfg" displayName="FMKIO_SerialCfg" ref="A34:F36" totalsRowShown="0">
-  <autoFilter ref="A34:F36" xr:uid="{978057A4-13F6-44F3-B65B-2C409866E1DE}"/>
-  <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{24FCFF33-29FB-4C97-8C6A-E82227514712}" name="Rx_GPIO_name"/>
-    <tableColumn id="4" xr3:uid="{12CA2E7A-25CB-4594-B099-0C3300125F20}" name="RxPin_name"/>
-    <tableColumn id="6" xr3:uid="{D003CF17-D1FC-4925-A150-971DDF359F41}" name="Tx_Gpio_Name"/>
-    <tableColumn id="5" xr3:uid="{14396C2C-537A-4355-B49A-DC2EB4D94AF0}" name="Tx_Pin_Name"/>
-    <tableColumn id="2" xr3:uid="{EBD561D8-5769-44A2-9D68-D1A8F057FDD0}" name="alternate function timer"/>
-    <tableColumn id="7" xr3:uid="{9DFBCFF1-0113-4C17-8011-2570BD8C9102}" name="UART/USART REF"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table25.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="32" xr:uid="{DA1831B2-BC94-42A9-B299-31A3CE618396}" name="FMKIO_IRQNHandler" displayName="FMKIO_IRQNHandler" ref="W29:W36" totalsRowShown="0">
-  <autoFilter ref="W29:W36" xr:uid="{DA1831B2-BC94-42A9-B299-31A3CE618396}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="32" xr:uid="{DA1831B2-BC94-42A9-B299-31A3CE618396}" name="FMKIO_IRQNHandler" displayName="FMKIO_IRQNHandler" ref="W28:W35" totalsRowShown="0">
+  <autoFilter ref="W28:W35" xr:uid="{DA1831B2-BC94-42A9-B299-31A3CE618396}"/>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{435A2CB3-E527-4D4E-9A3C-7D2BA856E09C}" name="List IRQN_Handler"/>
   </tableColumns>
@@ -4364,7 +4373,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table25.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{684AB3A4-4693-477C-AADC-64EBB335C3E9}" name="FMKTIM_EvntTimer" displayName="FMKTIM_EvntTimer" ref="B4:C6" totalsRowShown="0">
   <autoFilter ref="B4:C6" xr:uid="{684AB3A4-4693-477C-AADC-64EBB335C3E9}"/>
   <tableColumns count="2">
@@ -4375,7 +4384,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table26.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="31" xr:uid="{CCB68487-82CB-434C-A0E4-701B1FDDACF5}" name="FMKTIM_IRQNHandler" displayName="FMKTIM_IRQNHandler" ref="F4:G17" totalsRowShown="0">
   <autoFilter ref="F4:G17" xr:uid="{CCB68487-82CB-434C-A0E4-701B1FDDACF5}"/>
   <tableColumns count="2">
@@ -4386,7 +4395,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table28.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table27.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{953E7E02-522E-4F1F-B136-4D0BF069F045}" name="FMKHRT_IrqHandler" displayName="FMKHRT_IrqHandler" ref="Y5:Y12" totalsRowShown="0">
   <autoFilter ref="Y5:Y12" xr:uid="{953E7E02-522E-4F1F-B136-4D0BF069F045}"/>
   <tableColumns count="1">
@@ -4396,7 +4405,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table29.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table28.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="24" xr:uid="{A4F27ADC-56A6-479B-93EF-D6AA72368D72}" name="FMKCDA_CalibrationOthers" displayName="FMKCDA_CalibrationOthers" ref="I3:M6" totalsRowShown="0">
   <autoFilter ref="I3:M6" xr:uid="{A4F27ADC-56A6-479B-93EF-D6AA72368D72}"/>
   <tableColumns count="5">
@@ -4405,6 +4414,19 @@
     <tableColumn id="3" xr3:uid="{0793AAF2-321B-4695-AEBB-122FAB9D49F7}" name="Adc Vref"/>
     <tableColumn id="4" xr3:uid="{F1198D75-5BAD-4CA5-814F-DDA2BB66E5F2}" name="Channel Vref"/>
     <tableColumn id="5" xr3:uid="{6C202CA4-44FC-4E46-A4B5-AF7389AC3A4D}" name="Enable"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table29.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="25" xr:uid="{99B4503A-67B2-48AD-BE25-2B3425F892A9}" name="FMKCDA_VoltageRef" displayName="FMKCDA_VoltageRef" ref="T17:W22" totalsRowShown="0">
+  <autoFilter ref="T17:W22" xr:uid="{99B4503A-67B2-48AD-BE25-2B3425F892A9}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{0BCC2BC4-7FF0-4C14-809D-9D95A3225151}" name="Vref Calib"/>
+    <tableColumn id="2" xr3:uid="{0E78A6D4-DF9E-4966-A80E-64FE5BD9F1E2}" name="address  hexacecimal"/>
+    <tableColumn id="4" xr3:uid="{4C711A0D-EAF5-4229-B4D2-99254AE9F9BA}" name="Adc Vref"/>
+    <tableColumn id="5" xr3:uid="{0B4759AE-B188-4822-92BB-EEEB3203C895}" name="Channel Vref"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4422,19 +4444,6 @@
 </file>
 
 <file path=xl/tables/table30.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="25" xr:uid="{99B4503A-67B2-48AD-BE25-2B3425F892A9}" name="FMKCDA_VoltageRef" displayName="FMKCDA_VoltageRef" ref="T17:W22" totalsRowShown="0">
-  <autoFilter ref="T17:W22" xr:uid="{99B4503A-67B2-48AD-BE25-2B3425F892A9}"/>
-  <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{0BCC2BC4-7FF0-4C14-809D-9D95A3225151}" name="Vref Calib"/>
-    <tableColumn id="2" xr3:uid="{0E78A6D4-DF9E-4966-A80E-64FE5BD9F1E2}" name="address  hexacecimal"/>
-    <tableColumn id="4" xr3:uid="{4C711A0D-EAF5-4229-B4D2-99254AE9F9BA}" name="Adc Vref"/>
-    <tableColumn id="5" xr3:uid="{0B4759AE-B188-4822-92BB-EEEB3203C895}" name="Channel Vref"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table31.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="33" xr:uid="{FAF38277-E25D-413A-A145-AFBC74566FF1}" name="FMKCDA_IRQNHandler" displayName="FMKCDA_IRQNHandler" ref="E8:F12" totalsRowShown="0">
   <autoFilter ref="E8:F12" xr:uid="{FAF38277-E25D-413A-A145-AFBC74566FF1}"/>
   <tableColumns count="2">
@@ -4445,9 +4454,9 @@
 </table>
 </file>
 
-<file path=xl/tables/table32.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="29" xr:uid="{333A4E38-7E7A-4098-B282-4F58DD308AC2}" name="FMKMAC_Cfg" displayName="FMKMAC_Cfg" ref="B2:E14" totalsRowShown="0">
-  <autoFilter ref="B2:E14" xr:uid="{333A4E38-7E7A-4098-B282-4F58DD308AC2}"/>
+<file path=xl/tables/table31.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="29" xr:uid="{333A4E38-7E7A-4098-B282-4F58DD308AC2}" name="FMKMAC_Cfg" displayName="FMKMAC_Cfg" ref="B2:E16" totalsRowShown="0">
+  <autoFilter ref="B2:E16" xr:uid="{333A4E38-7E7A-4098-B282-4F58DD308AC2}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{9B6EDCAA-F526-412C-A8EC-AC6897A0EB04}" name="RqstDmaType"/>
     <tableColumn id="2" xr3:uid="{ED583461-6D2B-456F-A394-15F76B273D8C}" name="DMA "/>
@@ -4458,7 +4467,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table33.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table32.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="34" xr:uid="{8B613F4D-88F2-4091-AA3A-5550AB627653}" name="FMKMAC_IRQN" displayName="FMKMAC_IRQN" ref="J3:K18" totalsRowShown="0">
   <autoFilter ref="J3:K18" xr:uid="{8B613F4D-88F2-4091-AA3A-5550AB627653}"/>
   <tableColumns count="2">
@@ -4469,7 +4478,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table34.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table33.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="36" xr:uid="{9E75F4B3-8C66-44CB-A927-82E8A09563A2}" name="FMKMAC_DMAMUX" displayName="FMKMAC_DMAMUX" ref="P3:P4" totalsRowShown="0">
   <autoFilter ref="P3:P4" xr:uid="{9E75F4B3-8C66-44CB-A927-82E8A09563A2}"/>
   <tableColumns count="1">
@@ -4479,11 +4488,24 @@
 </table>
 </file>
 
-<file path=xl/tables/table35.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="35" xr:uid="{3568793B-2270-4B9A-A9E5-55F929444AFF}" name="Tableau35" displayName="Tableau35" ref="B5:B11" totalsRowShown="0">
+<file path=xl/tables/table34.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="35" xr:uid="{3568793B-2270-4B9A-A9E5-55F929444AFF}" name="fdcan_irqn_handler" displayName="fdcan_irqn_handler" ref="B5:B11" totalsRowShown="0">
   <autoFilter ref="B5:B11" xr:uid="{3568793B-2270-4B9A-A9E5-55F929444AFF}"/>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{61C0BDFB-C4E4-44F5-AA25-0ECEC1F95FDC}" name="List IRQN_Handler"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table35.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="38" xr:uid="{313ACF3F-AE43-48C2-87A6-B02CD6ECDE78}" name="Fdcan_Info" displayName="Fdcan_Info" ref="D5:G8" totalsRowShown="0">
+  <autoFilter ref="D5:G8" xr:uid="{313ACF3F-AE43-48C2-87A6-B02CD6ECDE78}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{972AC2AD-D7A3-42B3-A083-FAFBDC8C0BB5}" name="Instance"/>
+    <tableColumn id="4" xr3:uid="{DA881EFC-E0AA-4CA5-A828-AD294471ADF4}" name="RCC Clock"/>
+    <tableColumn id="2" xr3:uid="{D2D71E97-792B-48BD-B1F9-E06DA953DC08}" name="RxBuffer Size"/>
+    <tableColumn id="3" xr3:uid="{252CC4E1-9F08-4D67-A192-871597E2D59B}" name="Tx buffer Size"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4933,13 +4955,13 @@
   <sheetData>
     <row r="17" spans="1:30" x14ac:dyDescent="0.3">
       <c r="R17" t="s">
-        <v>458</v>
+        <v>455</v>
       </c>
       <c r="S17" t="s">
-        <v>459</v>
+        <v>456</v>
       </c>
       <c r="T17" t="s">
-        <v>460</v>
+        <v>457</v>
       </c>
     </row>
     <row r="18" spans="1:30" x14ac:dyDescent="0.3">
@@ -4953,7 +4975,7 @@
         <v>296</v>
       </c>
       <c r="F18" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
       <c r="H18" t="s">
         <v>57</v>
@@ -4997,7 +5019,7 @@
         <v>303</v>
       </c>
       <c r="F19" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H19" t="s">
         <v>59</v>
@@ -5029,7 +5051,7 @@
         <v>303</v>
       </c>
       <c r="F20" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H20" t="s">
         <v>124</v>
@@ -5070,7 +5092,7 @@
         <v>303</v>
       </c>
       <c r="F21" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H21" t="s">
         <v>125</v>
@@ -5111,7 +5133,7 @@
         <v>303</v>
       </c>
       <c r="F22" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H22" t="s">
         <v>126</v>
@@ -5152,7 +5174,7 @@
         <v>303</v>
       </c>
       <c r="F23" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H23" t="s">
         <v>60</v>
@@ -5184,7 +5206,7 @@
         <v>303</v>
       </c>
       <c r="F24" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H24" t="s">
         <v>61</v>
@@ -5216,7 +5238,7 @@
         <v>303</v>
       </c>
       <c r="F25" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H25" t="s">
         <v>127</v>
@@ -5248,7 +5270,7 @@
         <v>304</v>
       </c>
       <c r="F26" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H26" t="s">
         <v>128</v>
@@ -5286,7 +5308,7 @@
         <v>304</v>
       </c>
       <c r="F27" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H27" t="s">
         <v>129</v>
@@ -5324,7 +5346,7 @@
         <v>304</v>
       </c>
       <c r="F28" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H28" t="s">
         <v>130</v>
@@ -5362,7 +5384,7 @@
         <v>304</v>
       </c>
       <c r="F29" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H29" t="s">
         <v>131</v>
@@ -5394,7 +5416,7 @@
         <v>304</v>
       </c>
       <c r="F30" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H30" t="s">
         <v>62</v>
@@ -5426,7 +5448,7 @@
         <v>304</v>
       </c>
       <c r="F31" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H31" t="s">
         <v>132</v>
@@ -5443,7 +5465,7 @@
         <v>304</v>
       </c>
       <c r="F32" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H32" t="s">
         <v>133</v>
@@ -5460,7 +5482,7 @@
         <v>302</v>
       </c>
       <c r="F33" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="H33" t="s">
         <v>134</v>
@@ -5483,7 +5505,7 @@
         <v>302</v>
       </c>
       <c r="F34" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="H34" t="s">
         <v>135</v>
@@ -5506,7 +5528,7 @@
         <v>294</v>
       </c>
       <c r="F35" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H35" t="s">
         <v>136</v>
@@ -5529,7 +5551,7 @@
         <v>294</v>
       </c>
       <c r="F36" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H36" t="s">
         <v>137</v>
@@ -5558,7 +5580,7 @@
         <v>294</v>
       </c>
       <c r="F37" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H37" t="s">
         <v>138</v>
@@ -5587,7 +5609,7 @@
         <v>294</v>
       </c>
       <c r="F38" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H38" t="s">
         <v>139</v>
@@ -5610,7 +5632,7 @@
         <v>304</v>
       </c>
       <c r="F39" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H39" t="s">
         <v>140</v>
@@ -5633,7 +5655,7 @@
         <v>304</v>
       </c>
       <c r="F40" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H40" t="s">
         <v>141</v>
@@ -5660,7 +5682,7 @@
         <v>276</v>
       </c>
       <c r="Z40" t="s">
-        <v>481</v>
+        <v>477</v>
       </c>
       <c r="AG40" t="s">
         <v>88</v>
@@ -5674,7 +5696,7 @@
         <v>301</v>
       </c>
       <c r="F41" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="H41" t="s">
         <v>142</v>
@@ -5706,7 +5728,7 @@
         <v>293</v>
       </c>
       <c r="F42" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H42" t="s">
         <v>143</v>
@@ -5738,7 +5760,7 @@
         <v>293</v>
       </c>
       <c r="F43" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H43" t="s">
         <v>144</v>
@@ -5770,7 +5792,7 @@
         <v>293</v>
       </c>
       <c r="F44" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H44" t="s">
         <v>145</v>
@@ -5799,7 +5821,7 @@
         <v>293</v>
       </c>
       <c r="F45" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H45" t="s">
         <v>146</v>
@@ -5828,7 +5850,7 @@
         <v>293</v>
       </c>
       <c r="F46" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H46" t="s">
         <v>63</v>
@@ -5848,7 +5870,7 @@
         <v>293</v>
       </c>
       <c r="F47" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H47" t="s">
         <v>147</v>
@@ -5868,7 +5890,7 @@
         <v>293</v>
       </c>
       <c r="F48" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H48" t="s">
         <v>64</v>
@@ -5888,7 +5910,7 @@
         <v>293</v>
       </c>
       <c r="F49" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H49" t="s">
         <v>148</v>
@@ -5908,7 +5930,7 @@
         <v>293</v>
       </c>
       <c r="F50" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H50" t="s">
         <v>149</v>
@@ -5925,7 +5947,7 @@
         <v>293</v>
       </c>
       <c r="F51" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H51" t="s">
         <v>150</v>
@@ -5942,7 +5964,7 @@
         <v>293</v>
       </c>
       <c r="F52" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H52" t="s">
         <v>151</v>
@@ -5962,7 +5984,7 @@
         <v>293</v>
       </c>
       <c r="F53" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="H53" t="s">
         <v>152</v>
@@ -5982,7 +6004,7 @@
         <v>293</v>
       </c>
       <c r="F54" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="H54" t="s">
         <v>65</v>
@@ -6002,7 +6024,7 @@
         <v>293</v>
       </c>
       <c r="F55" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="H55" t="s">
         <v>66</v>
@@ -6022,7 +6044,7 @@
         <v>293</v>
       </c>
       <c r="F56" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="H56" t="s">
         <v>67</v>
@@ -6042,7 +6064,7 @@
         <v>293</v>
       </c>
       <c r="F57" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H57" t="s">
         <v>68</v>
@@ -6062,7 +6084,7 @@
         <v>293</v>
       </c>
       <c r="F58" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H58" t="s">
         <v>153</v>
@@ -6082,7 +6104,7 @@
         <v>301</v>
       </c>
       <c r="F59" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="H59" t="s">
         <v>154</v>
@@ -6102,7 +6124,7 @@
         <v>293</v>
       </c>
       <c r="F60" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H60" t="s">
         <v>155</v>
@@ -6122,7 +6144,7 @@
         <v>293</v>
       </c>
       <c r="F61" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="H61" t="s">
         <v>156</v>
@@ -6142,7 +6164,7 @@
         <v>293</v>
       </c>
       <c r="F62" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H62" t="s">
         <v>157</v>
@@ -6162,7 +6184,7 @@
         <v>293</v>
       </c>
       <c r="F63" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H63" t="s">
         <v>158</v>
@@ -6179,7 +6201,7 @@
         <v>294</v>
       </c>
       <c r="F64" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H64" t="s">
         <v>159</v>
@@ -6196,7 +6218,7 @@
         <v>294</v>
       </c>
       <c r="F65" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H65" t="s">
         <v>160</v>
@@ -6213,7 +6235,7 @@
         <v>294</v>
       </c>
       <c r="F66" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H66" t="s">
         <v>161</v>
@@ -6230,7 +6252,7 @@
         <v>294</v>
       </c>
       <c r="F67" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H67" t="s">
         <v>162</v>
@@ -6247,7 +6269,7 @@
         <v>294</v>
       </c>
       <c r="F68" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="H68" t="s">
         <v>163</v>
@@ -6264,7 +6286,7 @@
         <v>294</v>
       </c>
       <c r="F69" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H69" t="s">
         <v>164</v>
@@ -6281,7 +6303,7 @@
         <v>294</v>
       </c>
       <c r="F70" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H70" t="s">
         <v>165</v>
@@ -6298,7 +6320,7 @@
         <v>294</v>
       </c>
       <c r="F71" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H71" t="s">
         <v>166</v>
@@ -6315,7 +6337,7 @@
         <v>294</v>
       </c>
       <c r="F72" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H72" t="s">
         <v>167</v>
@@ -6332,13 +6354,13 @@
         <v>294</v>
       </c>
       <c r="F73" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H73" t="s">
         <v>168</v>
       </c>
       <c r="I73" t="s">
-        <v>69</v>
+        <v>90</v>
       </c>
     </row>
     <row r="74" spans="4:9" x14ac:dyDescent="0.3">
@@ -6349,7 +6371,7 @@
         <v>294</v>
       </c>
       <c r="F74" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H74" t="s">
         <v>169</v>
@@ -6366,7 +6388,7 @@
         <v>294</v>
       </c>
       <c r="F75" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H75" t="s">
         <v>170</v>
@@ -6774,18 +6796,18 @@
   <sheetData>
     <row r="3" spans="2:15" ht="93.6" x14ac:dyDescent="1.75">
       <c r="B3" s="6" t="s">
-        <v>436</v>
+        <v>433</v>
       </c>
     </row>
     <row r="5" spans="2:15" x14ac:dyDescent="0.3">
       <c r="J5" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
       <c r="K5" t="s">
-        <v>449</v>
+        <v>446</v>
       </c>
       <c r="L5" t="s">
-        <v>450</v>
+        <v>447</v>
       </c>
     </row>
     <row r="6" spans="2:15" x14ac:dyDescent="0.3">
@@ -6841,18 +6863,18 @@
     </row>
     <row r="20" spans="5:18" x14ac:dyDescent="0.3">
       <c r="E20" s="9" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
     </row>
     <row r="21" spans="5:18" x14ac:dyDescent="0.3">
       <c r="E21" s="7" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="F21" s="7">
         <f>$J$6 *$O$8 / $K$6</f>
@@ -6865,7 +6887,7 @@
     </row>
     <row r="22" spans="5:18" x14ac:dyDescent="0.3">
       <c r="E22" s="8" t="s">
-        <v>438</v>
+        <v>435</v>
       </c>
       <c r="F22" s="8">
         <f>$J$6 *$O$9 / $K$6</f>
@@ -6878,7 +6900,7 @@
     </row>
     <row r="23" spans="5:18" x14ac:dyDescent="0.3">
       <c r="E23" s="7" t="s">
-        <v>439</v>
+        <v>436</v>
       </c>
       <c r="F23" s="7">
         <f>$J$6 *$O$10 / $K$6</f>
@@ -6894,7 +6916,7 @@
     </row>
     <row r="24" spans="5:18" x14ac:dyDescent="0.3">
       <c r="E24" s="8" t="s">
-        <v>440</v>
+        <v>437</v>
       </c>
       <c r="F24" s="8">
         <f>$J$6 *$O$11 / $K$6</f>
@@ -6907,7 +6929,7 @@
     </row>
     <row r="25" spans="5:18" x14ac:dyDescent="0.3">
       <c r="E25" s="7" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="F25" s="7">
         <f>$J$6 *$O$12 / $K$6</f>
@@ -6920,7 +6942,7 @@
     </row>
     <row r="26" spans="5:18" x14ac:dyDescent="0.3">
       <c r="E26" s="8" t="s">
-        <v>442</v>
+        <v>439</v>
       </c>
       <c r="F26" s="8">
         <f>$J$6 *$O$13 / $K$6</f>
@@ -6933,7 +6955,7 @@
     </row>
     <row r="27" spans="5:18" x14ac:dyDescent="0.3">
       <c r="E27" s="7" t="s">
-        <v>443</v>
+        <v>440</v>
       </c>
       <c r="F27" s="7">
         <f>$J$6 / $O$14 / $K$6</f>
@@ -6946,7 +6968,7 @@
     </row>
     <row r="28" spans="5:18" x14ac:dyDescent="0.3">
       <c r="E28" s="11" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
       <c r="F28" s="11">
         <f>$J$6 / $O$15 / $K$6</f>
@@ -7002,10 +7024,10 @@
   <sheetData>
     <row r="2" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>435</v>
+        <v>432</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>434</v>
+        <v>431</v>
       </c>
     </row>
     <row r="5" spans="1:28" x14ac:dyDescent="0.3">
@@ -7081,7 +7103,7 @@
         <v>44</v>
       </c>
       <c r="U6" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="W6" t="s">
         <v>23</v>
@@ -7122,7 +7144,7 @@
         <v>31</v>
       </c>
       <c r="L7" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="M7" t="s">
         <v>252</v>
@@ -7137,7 +7159,7 @@
         <v>29</v>
       </c>
       <c r="R7" t="s">
-        <v>475</v>
+        <v>472</v>
       </c>
       <c r="S7" t="s">
         <v>7</v>
@@ -7146,7 +7168,7 @@
         <v>45</v>
       </c>
       <c r="U7" t="s">
-        <v>464</v>
+        <v>461</v>
       </c>
       <c r="W7" t="s">
         <v>12</v>
@@ -7155,7 +7177,7 @@
         <v>28</v>
       </c>
       <c r="Y7" t="s">
-        <v>478</v>
+        <v>475</v>
       </c>
       <c r="AA7" t="s">
         <v>23</v>
@@ -7190,7 +7212,7 @@
         <v>32</v>
       </c>
       <c r="L8" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="M8" t="s">
         <v>252</v>
@@ -7205,7 +7227,7 @@
         <v>34</v>
       </c>
       <c r="R8" t="s">
-        <v>476</v>
+        <v>473</v>
       </c>
       <c r="S8" t="s">
         <v>8</v>
@@ -7214,7 +7236,7 @@
         <v>45</v>
       </c>
       <c r="U8" t="s">
-        <v>464</v>
+        <v>461</v>
       </c>
       <c r="W8" t="s">
         <v>12</v>
@@ -7223,7 +7245,7 @@
         <v>30</v>
       </c>
       <c r="Y8" t="s">
-        <v>433</v>
+        <v>430</v>
       </c>
       <c r="AA8" t="s">
         <v>12</v>
@@ -7258,7 +7280,7 @@
         <v>38</v>
       </c>
       <c r="R9" t="s">
-        <v>474</v>
+        <v>471</v>
       </c>
       <c r="S9" t="s">
         <v>257</v>
@@ -7267,16 +7289,7 @@
         <v>46</v>
       </c>
       <c r="U9" t="s">
-        <v>464</v>
-      </c>
-      <c r="W9" t="s">
-        <v>13</v>
-      </c>
-      <c r="X9" t="s">
-        <v>29</v>
-      </c>
-      <c r="Y9" t="s">
-        <v>479</v>
+        <v>461</v>
       </c>
       <c r="AA9" t="s">
         <v>11</v>
@@ -7311,7 +7324,7 @@
         <v>41</v>
       </c>
       <c r="R10" t="s">
-        <v>477</v>
+        <v>474</v>
       </c>
       <c r="S10" t="s">
         <v>6</v>
@@ -7320,7 +7333,7 @@
         <v>46</v>
       </c>
       <c r="U10" t="s">
-        <v>464</v>
+        <v>461</v>
       </c>
       <c r="AA10" t="s">
         <v>11</v>
@@ -7355,7 +7368,7 @@
         <v>32</v>
       </c>
       <c r="R11" t="s">
-        <v>430</v>
+        <v>427</v>
       </c>
       <c r="S11" t="s">
         <v>255</v>
@@ -7364,7 +7377,7 @@
         <v>46</v>
       </c>
       <c r="U11" t="s">
-        <v>465</v>
+        <v>462</v>
       </c>
       <c r="AA11" t="s">
         <v>11</v>
@@ -7399,7 +7412,7 @@
         <v>27</v>
       </c>
       <c r="R12" t="s">
-        <v>473</v>
+        <v>470</v>
       </c>
       <c r="S12" t="s">
         <v>256</v>
@@ -7408,7 +7421,7 @@
         <v>45</v>
       </c>
       <c r="U12" t="s">
-        <v>465</v>
+        <v>462</v>
       </c>
       <c r="AA12" t="s">
         <v>12</v>
@@ -7431,7 +7444,7 @@
         <v>27</v>
       </c>
       <c r="R13" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
       <c r="S13" t="s">
         <v>4</v>
@@ -7440,7 +7453,7 @@
         <v>92</v>
       </c>
       <c r="U13" t="s">
-        <v>465</v>
+        <v>462</v>
       </c>
       <c r="AA13" t="s">
         <v>13</v>
@@ -7463,16 +7476,16 @@
         <v>33</v>
       </c>
       <c r="R14" s="7" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
       <c r="S14" s="7" t="s">
-        <v>463</v>
+        <v>460</v>
       </c>
       <c r="T14" s="7" t="s">
         <v>45</v>
       </c>
       <c r="U14" s="12" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
       <c r="AA14" t="s">
         <v>13</v>
@@ -7495,22 +7508,22 @@
         <v>35</v>
       </c>
       <c r="R15" s="8" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
       <c r="S15" s="8" t="s">
-        <v>467</v>
+        <v>464</v>
       </c>
       <c r="T15" s="8" t="s">
         <v>45</v>
       </c>
       <c r="U15" s="14" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
       <c r="AA15" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="AB15" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row r="16" spans="1:28" x14ac:dyDescent="0.3">
@@ -7521,22 +7534,22 @@
         <v>38</v>
       </c>
       <c r="R16" s="7" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
       <c r="S16" s="7" t="s">
-        <v>468</v>
+        <v>465</v>
       </c>
       <c r="T16" s="7" t="s">
         <v>45</v>
       </c>
       <c r="U16" s="12" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
       <c r="AA16" t="s">
         <v>15</v>
       </c>
       <c r="AB16" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="17" spans="1:53" x14ac:dyDescent="0.3">
@@ -7547,22 +7560,16 @@
         <v>40</v>
       </c>
       <c r="R17" s="8" t="s">
+        <v>463</v>
+      </c>
+      <c r="S17" s="8" t="s">
         <v>466</v>
-      </c>
-      <c r="S17" s="8" t="s">
-        <v>469</v>
       </c>
       <c r="T17" s="8" t="s">
         <v>45</v>
       </c>
       <c r="U17" s="14" t="s">
-        <v>462</v>
-      </c>
-      <c r="AA17" t="s">
-        <v>15</v>
-      </c>
-      <c r="AB17" t="s">
-        <v>26</v>
+        <v>459</v>
       </c>
     </row>
     <row r="18" spans="1:53" x14ac:dyDescent="0.3">
@@ -7573,16 +7580,16 @@
         <v>31</v>
       </c>
       <c r="R18" s="7" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
       <c r="S18" s="7" t="s">
-        <v>471</v>
+        <v>468</v>
       </c>
       <c r="T18" s="7" t="s">
         <v>45</v>
       </c>
       <c r="U18" s="12" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
     </row>
     <row r="19" spans="1:53" x14ac:dyDescent="0.3">
@@ -7593,21 +7600,21 @@
         <v>33</v>
       </c>
       <c r="R19" s="8" t="s">
-        <v>472</v>
+        <v>469</v>
       </c>
       <c r="S19" s="8" t="s">
-        <v>470</v>
+        <v>467</v>
       </c>
       <c r="T19" s="8" t="s">
         <v>45</v>
       </c>
       <c r="U19" s="14" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
     </row>
     <row r="24" spans="1:53" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
     </row>
     <row r="25" spans="1:53" x14ac:dyDescent="0.3">
@@ -7664,10 +7671,13 @@
         <v>41</v>
       </c>
       <c r="E27" t="s">
-        <v>283</v>
+        <v>490</v>
       </c>
       <c r="F27" t="s">
         <v>290</v>
+      </c>
+      <c r="W27" t="s">
+        <v>357</v>
       </c>
     </row>
     <row r="28" spans="1:53" x14ac:dyDescent="0.3">
@@ -7684,18 +7694,18 @@
         <v>38</v>
       </c>
       <c r="E28" t="s">
-        <v>283</v>
+        <v>494</v>
       </c>
       <c r="F28" t="s">
         <v>289</v>
       </c>
       <c r="W28" t="s">
-        <v>360</v>
+        <v>350</v>
       </c>
     </row>
     <row r="29" spans="1:53" x14ac:dyDescent="0.3">
       <c r="W29" t="s">
-        <v>353</v>
+        <v>358</v>
       </c>
       <c r="AW29" t="s">
         <v>91</v>
@@ -7706,7 +7716,7 @@
     </row>
     <row r="30" spans="1:53" x14ac:dyDescent="0.3">
       <c r="W30" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="AW30" t="s">
         <v>25</v>
@@ -7720,7 +7730,7 @@
     </row>
     <row r="31" spans="1:53" x14ac:dyDescent="0.3">
       <c r="W31" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="AW31" t="s">
         <v>26</v>
@@ -7734,7 +7744,7 @@
     </row>
     <row r="32" spans="1:53" x14ac:dyDescent="0.3">
       <c r="W32" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="AW32" t="s">
         <v>27</v>
@@ -7746,12 +7756,9 @@
         <v>96</v>
       </c>
     </row>
-    <row r="33" spans="1:53" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
-        <v>343</v>
-      </c>
+    <row r="33" spans="23:53" x14ac:dyDescent="0.3">
       <c r="W33" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="AW33" t="s">
         <v>28</v>
@@ -7763,27 +7770,9 @@
         <v>97</v>
       </c>
     </row>
-    <row r="34" spans="1:53" x14ac:dyDescent="0.3">
-      <c r="A34" t="s">
-        <v>284</v>
-      </c>
-      <c r="B34" t="s">
-        <v>285</v>
-      </c>
-      <c r="C34" t="s">
-        <v>286</v>
-      </c>
-      <c r="D34" t="s">
-        <v>287</v>
-      </c>
-      <c r="E34" t="s">
-        <v>42</v>
-      </c>
-      <c r="F34" t="s">
-        <v>346</v>
-      </c>
+    <row r="34" spans="23:53" x14ac:dyDescent="0.3">
       <c r="W34" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="AW34" t="s">
         <v>29</v>
@@ -7795,27 +7784,9 @@
         <v>98</v>
       </c>
     </row>
-    <row r="35" spans="1:53" x14ac:dyDescent="0.3">
-      <c r="A35" t="s">
-        <v>11</v>
-      </c>
-      <c r="B35" t="s">
-        <v>28</v>
-      </c>
-      <c r="C35" t="s">
-        <v>11</v>
-      </c>
-      <c r="D35" t="s">
-        <v>27</v>
-      </c>
-      <c r="E35" t="s">
-        <v>344</v>
-      </c>
-      <c r="F35" t="s">
-        <v>79</v>
-      </c>
+    <row r="35" spans="23:53" x14ac:dyDescent="0.3">
       <c r="W35" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="AW35" t="s">
         <v>30</v>
@@ -7824,28 +7795,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="36" spans="1:53" x14ac:dyDescent="0.3">
-      <c r="A36" t="s">
-        <v>13</v>
-      </c>
-      <c r="B36" t="s">
-        <v>36</v>
-      </c>
-      <c r="C36" t="s">
-        <v>13</v>
-      </c>
-      <c r="D36" t="s">
-        <v>35</v>
-      </c>
-      <c r="E36" t="s">
-        <v>345</v>
-      </c>
-      <c r="F36" t="s">
-        <v>277</v>
-      </c>
-      <c r="W36" t="s">
-        <v>367</v>
-      </c>
+    <row r="36" spans="23:53" x14ac:dyDescent="0.3">
       <c r="AW36" t="s">
         <v>31</v>
       </c>
@@ -7853,7 +7803,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="37" spans="1:53" x14ac:dyDescent="0.3">
+    <row r="37" spans="23:53" x14ac:dyDescent="0.3">
       <c r="AW37" t="s">
         <v>32</v>
       </c>
@@ -7861,7 +7811,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="38" spans="1:53" x14ac:dyDescent="0.3">
+    <row r="38" spans="23:53" x14ac:dyDescent="0.3">
       <c r="AW38" t="s">
         <v>33</v>
       </c>
@@ -7869,7 +7819,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="39" spans="1:53" x14ac:dyDescent="0.3">
+    <row r="39" spans="23:53" x14ac:dyDescent="0.3">
       <c r="AW39" t="s">
         <v>34</v>
       </c>
@@ -7877,7 +7827,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="40" spans="1:53" x14ac:dyDescent="0.3">
+    <row r="40" spans="23:53" x14ac:dyDescent="0.3">
       <c r="AW40" t="s">
         <v>35</v>
       </c>
@@ -7885,7 +7835,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="41" spans="1:53" x14ac:dyDescent="0.3">
+    <row r="41" spans="23:53" x14ac:dyDescent="0.3">
       <c r="AW41" t="s">
         <v>36</v>
       </c>
@@ -7893,7 +7843,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="42" spans="1:53" x14ac:dyDescent="0.3">
+    <row r="42" spans="23:53" x14ac:dyDescent="0.3">
       <c r="AW42" t="s">
         <v>38</v>
       </c>
@@ -7901,7 +7851,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="43" spans="1:53" x14ac:dyDescent="0.3">
+    <row r="43" spans="23:53" x14ac:dyDescent="0.3">
       <c r="AW43" t="s">
         <v>39</v>
       </c>
@@ -7909,7 +7859,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="44" spans="1:53" x14ac:dyDescent="0.3">
+    <row r="44" spans="23:53" x14ac:dyDescent="0.3">
       <c r="AW44" t="s">
         <v>40</v>
       </c>
@@ -7917,7 +7867,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="45" spans="1:53" x14ac:dyDescent="0.3">
+    <row r="45" spans="23:53" x14ac:dyDescent="0.3">
       <c r="AW45" t="s">
         <v>41</v>
       </c>
@@ -7925,19 +7875,19 @@
         <v>109</v>
       </c>
     </row>
-    <row r="46" spans="1:53" x14ac:dyDescent="0.3">
+    <row r="46" spans="23:53" x14ac:dyDescent="0.3">
       <c r="BA46" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="47" spans="1:53" x14ac:dyDescent="0.3">
+    <row r="47" spans="23:53" x14ac:dyDescent="0.3">
       <c r="BA47" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="48" spans="1:53" x14ac:dyDescent="0.3">
+    <row r="48" spans="23:53" x14ac:dyDescent="0.3">
       <c r="BA48" t="s">
-        <v>480</v>
+        <v>476</v>
       </c>
     </row>
     <row r="57" spans="36:36" x14ac:dyDescent="0.3">
@@ -7948,7 +7898,7 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <dataValidations count="5">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AW46 Q14:Q19 Q7 B7:B15 X7:X9 AB15:AB16 K7:K8 AB8:AB13 F7:F12" xr:uid="{14BC2D73-1395-4E2C-9D1E-55C781825C64}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AW46 Q14:Q19 Q7 B7:B15 X7:X8 K7:K8 AB8:AB13 F7:F12 AB15" xr:uid="{14BC2D73-1395-4E2C-9D1E-55C781825C64}">
       <formula1>$AW$30:$AW$45</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="T14:T19 T7 N7:N8" xr:uid="{727A5344-B28A-4866-9EC1-7C96029AF8B6}">
@@ -7966,7 +7916,7 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-  <tableParts count="12">
+  <tableParts count="11">
     <tablePart r:id="rId2"/>
     <tablePart r:id="rId3"/>
     <tablePart r:id="rId4"/>
@@ -7978,7 +7928,6 @@
     <tablePart r:id="rId10"/>
     <tablePart r:id="rId11"/>
     <tablePart r:id="rId12"/>
-    <tablePart r:id="rId13"/>
   </tableParts>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
@@ -7987,7 +7936,7 @@
           <x14:formula1>
             <xm:f>General_Info!$P$34:$P$39</xm:f>
           </x14:formula1>
-          <xm:sqref>P14:P19 P7 A7:A15 W7:W9 AA15:AA16 J7:J8 AA8:AA13 E7:E12</xm:sqref>
+          <xm:sqref>P14:P19 P7 A7:A15 W7:W8 J7:J8 AA8:AA13 E7:E12 AA15</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{3C428027-B16D-4B04-9CB2-8290577ED0FB}">
           <x14:formula1>
@@ -8017,7 +7966,7 @@
         <v>51</v>
       </c>
       <c r="F3" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.3">
@@ -8028,10 +7977,10 @@
         <v>1</v>
       </c>
       <c r="F4" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="G4" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.3">
@@ -8042,7 +7991,7 @@
         <v>45</v>
       </c>
       <c r="F5" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="G5" t="s">
         <v>6</v>
@@ -8056,7 +8005,7 @@
         <v>45</v>
       </c>
       <c r="F6" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
       <c r="G6" t="s">
         <v>7</v>
@@ -8064,7 +8013,7 @@
     </row>
     <row r="7" spans="2:7" x14ac:dyDescent="0.3">
       <c r="F7" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="G7" t="s">
         <v>8</v>
@@ -8072,7 +8021,7 @@
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.3">
       <c r="F8" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="G8" t="s">
         <v>4</v>
@@ -8080,7 +8029,7 @@
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.3">
       <c r="F9" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="G9" t="s">
         <v>251</v>
@@ -8088,7 +8037,7 @@
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.3">
       <c r="F10" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="G10" t="s">
         <v>5</v>
@@ -8096,7 +8045,7 @@
     </row>
     <row r="11" spans="2:7" x14ac:dyDescent="0.3">
       <c r="F11" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="G11" t="s">
         <v>252</v>
@@ -8104,7 +8053,7 @@
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.3">
       <c r="F12" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="G12" t="s">
         <v>253</v>
@@ -8112,7 +8061,7 @@
     </row>
     <row r="13" spans="2:7" x14ac:dyDescent="0.3">
       <c r="F13" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="G13" t="s">
         <v>254</v>
@@ -8120,7 +8069,7 @@
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.3">
       <c r="F14" t="s">
-        <v>432</v>
+        <v>429</v>
       </c>
       <c r="G14" t="s">
         <v>255</v>
@@ -8128,7 +8077,7 @@
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.3">
       <c r="F15" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
       <c r="G15" t="s">
         <v>256</v>
@@ -8136,7 +8085,7 @@
     </row>
     <row r="16" spans="2:7" x14ac:dyDescent="0.3">
       <c r="F16" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="G16" t="s">
         <v>256</v>
@@ -8144,7 +8093,7 @@
     </row>
     <row r="17" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F17" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="G17" t="s">
         <v>256</v>
@@ -8175,37 +8124,37 @@
     </row>
     <row r="6" spans="25:25" x14ac:dyDescent="0.3">
       <c r="Y6" t="s">
-        <v>453</v>
+        <v>450</v>
       </c>
     </row>
     <row r="7" spans="25:25" x14ac:dyDescent="0.3">
       <c r="Y7" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
     </row>
     <row r="8" spans="25:25" x14ac:dyDescent="0.3">
       <c r="Y8" t="s">
-        <v>454</v>
+        <v>451</v>
       </c>
     </row>
     <row r="9" spans="25:25" x14ac:dyDescent="0.3">
       <c r="Y9" t="s">
-        <v>451</v>
+        <v>448</v>
       </c>
     </row>
     <row r="10" spans="25:25" x14ac:dyDescent="0.3">
       <c r="Y10" t="s">
-        <v>455</v>
+        <v>452</v>
       </c>
     </row>
     <row r="11" spans="25:25" x14ac:dyDescent="0.3">
       <c r="Y11" t="s">
-        <v>456</v>
+        <v>453</v>
       </c>
     </row>
     <row r="12" spans="25:25" x14ac:dyDescent="0.3">
       <c r="Y12" t="s">
-        <v>457</v>
+        <v>454</v>
       </c>
     </row>
   </sheetData>
@@ -8256,15 +8205,15 @@
         <v>119</v>
       </c>
       <c r="M3" t="s">
-        <v>484</v>
+        <v>480</v>
       </c>
     </row>
     <row r="4" spans="5:17" x14ac:dyDescent="0.3">
       <c r="I4" t="s">
-        <v>482</v>
+        <v>478</v>
       </c>
       <c r="J4" t="s">
-        <v>483</v>
+        <v>479</v>
       </c>
       <c r="K4" t="s">
         <v>16</v>
@@ -8273,7 +8222,7 @@
         <v>111</v>
       </c>
       <c r="M4" t="s">
-        <v>485</v>
+        <v>481</v>
       </c>
     </row>
     <row r="5" spans="5:17" x14ac:dyDescent="0.3">
@@ -8290,7 +8239,7 @@
         <v>110</v>
       </c>
       <c r="M5" t="s">
-        <v>486</v>
+        <v>481</v>
       </c>
     </row>
     <row r="6" spans="5:17" x14ac:dyDescent="0.3">
@@ -8307,52 +8256,52 @@
         <v>98</v>
       </c>
       <c r="M6" t="s">
-        <v>486</v>
+        <v>482</v>
       </c>
     </row>
     <row r="7" spans="5:17" x14ac:dyDescent="0.3">
       <c r="E7" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
     </row>
     <row r="8" spans="5:17" x14ac:dyDescent="0.3">
       <c r="E8" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="F8" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
     </row>
     <row r="9" spans="5:17" x14ac:dyDescent="0.3">
       <c r="E9" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="F9" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
     </row>
     <row r="10" spans="5:17" x14ac:dyDescent="0.3">
       <c r="E10" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="F10" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
     </row>
     <row r="11" spans="5:17" x14ac:dyDescent="0.3">
       <c r="E11" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="F11" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
     </row>
     <row r="12" spans="5:17" x14ac:dyDescent="0.3">
       <c r="E12" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="F12" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
     </row>
     <row r="17" spans="20:23" x14ac:dyDescent="0.3">
@@ -8371,7 +8320,7 @@
     </row>
     <row r="18" spans="20:23" x14ac:dyDescent="0.3">
       <c r="T18" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="U18" t="s">
         <v>268</v>
@@ -8380,12 +8329,12 @@
         <v>16</v>
       </c>
       <c r="W18" t="s">
-        <v>480</v>
+        <v>476</v>
       </c>
     </row>
     <row r="19" spans="20:23" x14ac:dyDescent="0.3">
       <c r="T19" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
       <c r="U19" t="s">
         <v>268</v>
@@ -8394,12 +8343,12 @@
         <v>16</v>
       </c>
       <c r="W19" t="s">
-        <v>480</v>
+        <v>476</v>
       </c>
     </row>
     <row r="20" spans="20:23" x14ac:dyDescent="0.3">
       <c r="T20" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="U20" t="s">
         <v>268</v>
@@ -8408,12 +8357,12 @@
         <v>262</v>
       </c>
       <c r="W20" t="s">
-        <v>480</v>
+        <v>476</v>
       </c>
     </row>
     <row r="21" spans="20:23" x14ac:dyDescent="0.3">
       <c r="T21" t="s">
-        <v>422</v>
+        <v>419</v>
       </c>
       <c r="U21" t="s">
         <v>268</v>
@@ -8422,12 +8371,12 @@
         <v>263</v>
       </c>
       <c r="W21" t="s">
-        <v>480</v>
+        <v>476</v>
       </c>
     </row>
     <row r="22" spans="20:23" x14ac:dyDescent="0.3">
       <c r="T22" t="s">
-        <v>423</v>
+        <v>420</v>
       </c>
       <c r="U22" t="s">
         <v>268</v>
@@ -8436,7 +8385,7 @@
         <v>264</v>
       </c>
       <c r="W22" t="s">
-        <v>480</v>
+        <v>476</v>
       </c>
     </row>
   </sheetData>
@@ -8470,7 +8419,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06E18236-E25D-41B3-8B1E-0194276152B3}">
-  <dimension ref="B2:P18"/>
+  <dimension ref="B1:P18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="19.33203125" customWidth="1"/>
@@ -8481,6 +8430,11 @@
     <col min="16" max="16" width="25.33203125" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="1" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B1" t="s">
+        <v>493</v>
+      </c>
+    </row>
     <row r="2" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
         <v>332</v>
@@ -8495,7 +8449,7 @@
         <v>335</v>
       </c>
       <c r="J2" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
     </row>
     <row r="3" spans="2:16" x14ac:dyDescent="0.3">
@@ -8512,18 +8466,18 @@
         <v>69</v>
       </c>
       <c r="J3" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="K3" t="s">
+        <v>402</v>
+      </c>
+      <c r="P3" t="s">
         <v>405</v>
-      </c>
-      <c r="P3" t="s">
-        <v>408</v>
       </c>
     </row>
     <row r="4" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="C4" t="s">
         <v>330</v>
@@ -8535,13 +8489,13 @@
         <v>69</v>
       </c>
       <c r="J4" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="K4" t="s">
         <v>329</v>
       </c>
       <c r="L4" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
       <c r="P4" t="s">
         <v>233</v>
@@ -8549,7 +8503,7 @@
     </row>
     <row r="5" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="C5" t="s">
         <v>330</v>
@@ -8561,15 +8515,15 @@
         <v>69</v>
       </c>
       <c r="J5" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="K5" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
     </row>
     <row r="6" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
       <c r="C6" t="s">
         <v>331</v>
@@ -8581,15 +8535,15 @@
         <v>69</v>
       </c>
       <c r="J6" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="K6" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
     </row>
     <row r="7" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
       <c r="C7" t="s">
         <v>331</v>
@@ -8601,7 +8555,7 @@
         <v>69</v>
       </c>
       <c r="J7" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="K7" t="s">
         <v>337</v>
@@ -8621,7 +8575,7 @@
         <v>69</v>
       </c>
       <c r="J8" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="K8" t="s">
         <v>338</v>
@@ -8641,7 +8595,7 @@
         <v>69</v>
       </c>
       <c r="J9" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="K9" t="s">
         <v>339</v>
@@ -8661,7 +8615,7 @@
         <v>69</v>
       </c>
       <c r="J10" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
       <c r="K10" t="s">
         <v>341</v>
@@ -8681,15 +8635,15 @@
         <v>69</v>
       </c>
       <c r="J11" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="K11" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
     </row>
     <row r="12" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B12" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="C12" t="s">
         <v>330</v>
@@ -8701,15 +8655,15 @@
         <v>69</v>
       </c>
       <c r="J12" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
       <c r="K12" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
     </row>
     <row r="13" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B13" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="C13" t="s">
         <v>330</v>
@@ -8721,47 +8675,77 @@
         <v>69</v>
       </c>
       <c r="J13" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
       <c r="K13" t="s">
-        <v>428</v>
+        <v>425</v>
       </c>
     </row>
     <row r="14" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B14" t="s">
-        <v>428</v>
+        <v>491</v>
       </c>
       <c r="C14" t="s">
         <v>331</v>
       </c>
       <c r="D14" t="s">
+        <v>340</v>
+      </c>
+      <c r="E14" t="s">
+        <v>69</v>
+      </c>
+      <c r="J14" t="s">
+        <v>379</v>
+      </c>
+      <c r="K14" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="15" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B15" t="s">
+        <v>492</v>
+      </c>
+      <c r="C15" t="s">
+        <v>331</v>
+      </c>
+      <c r="D15" t="s">
+        <v>342</v>
+      </c>
+      <c r="E15" t="s">
+        <v>69</v>
+      </c>
+      <c r="J15" t="s">
+        <v>380</v>
+      </c>
+      <c r="K15" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="16" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B16" t="s">
+        <v>425</v>
+      </c>
+      <c r="C16" t="s">
+        <v>331</v>
+      </c>
+      <c r="D16" t="s">
         <v>92</v>
       </c>
-      <c r="E14" s="4" t="s">
+      <c r="E16" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="J14" t="s">
-        <v>382</v>
-      </c>
-    </row>
-    <row r="15" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="J15" t="s">
-        <v>383</v>
-      </c>
-    </row>
-    <row r="16" spans="2:16" x14ac:dyDescent="0.3">
       <c r="J16" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
     </row>
     <row r="17" spans="10:10" x14ac:dyDescent="0.3">
       <c r="J17" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
     </row>
     <row r="18" spans="10:10" x14ac:dyDescent="0.3">
       <c r="J18" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
     </row>
   </sheetData>
@@ -8776,58 +8760,112 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9D1D4C8-FD0D-4DBE-B311-5297C41CC83F}">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="23.77734375" customWidth="1"/>
+    <col min="6" max="6" width="25" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B4" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B5" t="s">
+        <v>350</v>
+      </c>
+      <c r="D5" t="s">
+        <v>483</v>
+      </c>
+      <c r="E5" t="s">
+        <v>489</v>
+      </c>
+      <c r="F5" t="s">
+        <v>485</v>
+      </c>
+      <c r="G5" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B6" t="s">
+        <v>385</v>
+      </c>
+      <c r="D6" t="s">
+        <v>484</v>
+      </c>
+      <c r="E6" t="s">
+        <v>246</v>
+      </c>
+      <c r="F6">
+        <v>40</v>
+      </c>
+      <c r="G6">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B7" t="s">
+        <v>386</v>
+      </c>
+      <c r="D7" t="s">
+        <v>487</v>
+      </c>
+      <c r="E7" t="s">
+        <v>246</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B8" t="s">
         <v>387</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B4" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B5" t="s">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B6" t="s">
+      <c r="D8" t="s">
+        <v>488</v>
+      </c>
+      <c r="E8" t="s">
+        <v>246</v>
+      </c>
+      <c r="F8">
+        <v>0</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B9" t="s">
         <v>388</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B7" t="s">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B10" t="s">
         <v>389</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B8" t="s">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B11" t="s">
         <v>390</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B9" t="s">
-        <v>391</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B10" t="s">
-        <v>392</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B11" t="s">
-        <v>393</v>
-      </c>
-    </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
+  <tableParts count="2">
     <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
@@ -8851,16 +8889,16 @@
   <sheetData>
     <row r="2" spans="5:13" x14ac:dyDescent="0.3">
       <c r="E2" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="F2" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="G2" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
       <c r="H2" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
       <c r="I2" t="s">
         <v>284</v>
@@ -8883,28 +8921,28 @@
         <v>78</v>
       </c>
       <c r="F3" t="s">
-        <v>412</v>
+        <v>409</v>
       </c>
       <c r="G3">
-        <v>0</v>
+        <v>256</v>
       </c>
       <c r="H3">
-        <v>0</v>
+        <v>256</v>
       </c>
       <c r="I3" t="s">
-        <v>259</v>
+        <v>13</v>
       </c>
       <c r="J3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="K3" t="s">
-        <v>259</v>
+        <v>13</v>
       </c>
       <c r="L3" t="s">
         <v>29</v>
       </c>
       <c r="M3" t="s">
-        <v>424</v>
+        <v>421</v>
       </c>
     </row>
     <row r="4" spans="5:13" x14ac:dyDescent="0.3">
@@ -8912,7 +8950,7 @@
         <v>79</v>
       </c>
       <c r="F4" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
       <c r="G4">
         <v>256</v>
@@ -8933,7 +8971,7 @@
         <v>27</v>
       </c>
       <c r="M4" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="5" spans="5:13" x14ac:dyDescent="0.3">
@@ -8941,7 +8979,13 @@
         <v>219</v>
       </c>
       <c r="F5" t="s">
-        <v>414</v>
+        <v>411</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
       </c>
       <c r="I5" t="s">
         <v>259</v>
@@ -8956,7 +9000,7 @@
         <v>31</v>
       </c>
       <c r="M5" t="s">
-        <v>425</v>
+        <v>422</v>
       </c>
     </row>
     <row r="6" spans="5:13" x14ac:dyDescent="0.3">
@@ -8964,13 +9008,13 @@
         <v>277</v>
       </c>
       <c r="F6" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="G6">
-        <v>256</v>
+        <v>0</v>
       </c>
       <c r="H6">
-        <v>256</v>
+        <v>0</v>
       </c>
       <c r="I6" t="s">
         <v>259</v>
@@ -8985,7 +9029,7 @@
         <v>33</v>
       </c>
       <c r="M6" t="s">
-        <v>427</v>
+        <v>424</v>
       </c>
     </row>
     <row r="7" spans="5:13" x14ac:dyDescent="0.3">
@@ -8993,7 +9037,7 @@
         <v>278</v>
       </c>
       <c r="F7" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="G7">
         <v>0</v>
@@ -9014,7 +9058,7 @@
         <v>35</v>
       </c>
       <c r="M7" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add watchdogs & pid library
</commit_message>
<xml_diff>
--- a/Doc/ConfigPrj/ExcelCfg/STM32G474RE/STM32G474RE_HwCfg.xlsx
+++ b/Doc/ConfigPrj/ExcelCfg/STM32G474RE/STM32G474RE_HwCfg.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\Software\STM32\Gamma_fCreateCfg\Doc\ConfigPrj\ExcelCfg\STM32G474RE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2BD330D-240E-41F1-9514-7F79FA8EA4DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A78DB2E-38D7-45E8-A6D6-F93AA8ED9B2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="7" xr2:uid="{2AF09063-600F-437A-B138-F66136E922A5}"/>
   </bookViews>
@@ -8953,10 +8953,10 @@
         <v>410</v>
       </c>
       <c r="G4">
-        <v>256</v>
+        <v>0</v>
       </c>
       <c r="H4">
-        <v>256</v>
+        <v>1024</v>
       </c>
       <c r="I4" t="s">
         <v>11</v>

</xml_diff>

<commit_message>
inout frequency tested and working as fuch
add safemme in FMKIO & FMKTIM
frequency pwm working
</commit_message>
<xml_diff>
--- a/Doc/ConfigPrj/ExcelCfg/STM32G474RE/STM32G474RE_HwCfg.xlsx
+++ b/Doc/ConfigPrj/ExcelCfg/STM32G474RE/STM32G474RE_HwCfg.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\Software\STM32\Gamma_fCreateCfg\Doc\ConfigPrj\ExcelCfg\STM32G474RE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A628473-AC41-43E3-8D8C-E93CAB3108BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70F47A61-A112-45B9-9ADF-2787DBF4B01E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="7" xr2:uid="{2AF09063-600F-437A-B138-F66136E922A5}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="8" xr2:uid="{2AF09063-600F-437A-B138-F66136E922A5}"/>
   </bookViews>
   <sheets>
     <sheet name="General_Info" sheetId="1" r:id="rId1"/>
@@ -3529,6 +3529,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="zero"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -3536,7 +3537,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -9103,7 +9103,7 @@
     </row>
     <row r="5" spans="3:14" x14ac:dyDescent="0.3">
       <c r="L5">
-        <v>21332.3</v>
+        <v>65000</v>
       </c>
       <c r="N5">
         <v>9</v>
@@ -9128,21 +9128,20 @@
     </row>
     <row r="8" spans="3:14" x14ac:dyDescent="0.3">
       <c r="D8">
-        <v>6000</v>
+        <v>8000</v>
       </c>
       <c r="E8">
         <v>128</v>
       </c>
       <c r="F8">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G8">
-        <f>E8*C3/((D8)*(F8+1))-1</f>
-        <v>21332.333333333332</v>
+        <v>50195</v>
       </c>
       <c r="J8">
         <f>(E8*1000000)/((L5))</f>
-        <v>6000.2906390778307</v>
+        <v>1969.2307692307693</v>
       </c>
       <c r="M8" t="s">
         <v>316</v>
@@ -9151,43 +9150,43 @@
     <row r="9" spans="3:14" x14ac:dyDescent="0.3">
       <c r="M9">
         <f>J14-ROUND(J14,0)</f>
-        <v>4.8439846304981771E-5</v>
+        <v>0.24615384615384617</v>
       </c>
     </row>
     <row r="12" spans="3:14" x14ac:dyDescent="0.3">
+      <c r="D12">
+        <f>(E8*C3)/((F8+1)*(G8+1))</f>
+        <v>850.00132812707523</v>
+      </c>
       <c r="L12" t="s">
         <v>315</v>
       </c>
     </row>
     <row r="13" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="D13">
-        <f>E8/(L13+1)*D8</f>
-        <v>35.998312579097856</v>
-      </c>
       <c r="J13" t="s">
         <v>311</v>
       </c>
-      <c r="L13">
+      <c r="L13" t="e">
         <f>L5+(L5/J15)*M9</f>
-        <v>21333.333333333332</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="14" spans="3:14" x14ac:dyDescent="0.3">
       <c r="J14">
         <f>E8*C3/(D8*(L5))</f>
-        <v>1.000048439846305</v>
+        <v>0.24615384615384617</v>
       </c>
     </row>
     <row r="15" spans="3:14" x14ac:dyDescent="0.3">
       <c r="J15">
         <f>TRUNC(J14)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="3:14" x14ac:dyDescent="0.3">
       <c r="D16">
         <f>E8*C3/D8</f>
-        <v>21333.333333333332</v>
+        <v>16000</v>
       </c>
       <c r="J16" t="s">
         <v>112</v>
@@ -9204,15 +9203,15 @@
     <row r="18" spans="2:16" x14ac:dyDescent="0.3">
       <c r="D18">
         <f>E8*C3/D16</f>
-        <v>6000</v>
+        <v>8000</v>
       </c>
       <c r="J18">
         <f>(E8*C3)/((L5)*(INT(J14)+1))</f>
-        <v>3000.1453195389154</v>
-      </c>
-      <c r="L18">
+        <v>1969.2307692307693</v>
+      </c>
+      <c r="L18" t="e">
         <f>(E8*C3)/((J15)*(L13))</f>
-        <v>6000</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="23" spans="2:16" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
end working on framework, we leave it that way for now, i think everythin is working, will have to check pwm, but freq, ana works
</commit_message>
<xml_diff>
--- a/Doc/ConfigPrj/ExcelCfg/STM32G474RE/STM32G474RE_HwCfg.xlsx
+++ b/Doc/ConfigPrj/ExcelCfg/STM32G474RE/STM32G474RE_HwCfg.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\Software\STM32\Gamma_fCreateCfg\Doc\ConfigPrj\ExcelCfg\STM32G474RE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70F47A61-A112-45B9-9ADF-2787DBF4B01E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{067BA571-2B01-4CF8-A8D9-FA6606A17F16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="8" xr2:uid="{2AF09063-600F-437A-B138-F66136E922A5}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="7" activeTab="9" xr2:uid="{2AF09063-600F-437A-B138-F66136E922A5}"/>
   </bookViews>
   <sheets>
     <sheet name="General_Info" sheetId="1" r:id="rId1"/>
@@ -9134,10 +9134,10 @@
         <v>128</v>
       </c>
       <c r="F8">
-        <v>2</v>
+        <v>62</v>
       </c>
       <c r="G8">
-        <v>50195</v>
+        <v>50793</v>
       </c>
       <c r="J8">
         <f>(E8*1000000)/((L5))</f>
@@ -9156,7 +9156,7 @@
     <row r="12" spans="3:14" x14ac:dyDescent="0.3">
       <c r="D12">
         <f>(E8*C3)/((F8+1)*(G8+1))</f>
-        <v>850.00132812707523</v>
+        <v>39.99972500189061</v>
       </c>
       <c r="L12" t="s">
         <v>315</v>

</xml_diff>

<commit_message>
Calibration worling when calibration not suppose to work^^
set algo param OK
</commit_message>
<xml_diff>
--- a/Doc/ConfigPrj/ExcelCfg/STM32G474RE/STM32G474RE_HwCfg.xlsx
+++ b/Doc/ConfigPrj/ExcelCfg/STM32G474RE/STM32G474RE_HwCfg.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\Software\STM32\Gamma_fMotionPlanner\Doc\ConfigPrj\ExcelCfg\STM32G474RE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36BA9811-3D8F-4240-B01B-2F2FA18A644F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A89548D-74B4-4D20-9AC0-4ABADB2625EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="1" xr2:uid="{2AF09063-600F-437A-B138-F66136E922A5}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{2AF09063-600F-437A-B138-F66136E922A5}"/>
   </bookViews>
   <sheets>
     <sheet name="General_Info" sheetId="1" r:id="rId1"/>
@@ -5590,7 +5590,7 @@
         <v>143</v>
       </c>
       <c r="N28" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="O28" t="s">
         <v>291</v>

</xml_diff>

<commit_message>
gantry perfectly synchronize for same x,y,z position but not whenever the position are short and long because of the nature of CL42T driver, to improve
</commit_message>
<xml_diff>
--- a/Doc/ConfigPrj/ExcelCfg/STM32G474RE/STM32G474RE_HwCfg.xlsx
+++ b/Doc/ConfigPrj/ExcelCfg/STM32G474RE/STM32G474RE_HwCfg.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\Software\STM32\Gamma_fMotionPlanner\Doc\ConfigPrj\ExcelCfg\STM32G474RE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A89548D-74B4-4D20-9AC0-4ABADB2625EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0C2792E-3412-4261-8C95-67427E1660E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{2AF09063-600F-437A-B138-F66136E922A5}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2AF09063-600F-437A-B138-F66136E922A5}"/>
   </bookViews>
   <sheets>
     <sheet name="General_Info" sheetId="1" r:id="rId1"/>
@@ -5590,7 +5590,7 @@
         <v>143</v>
       </c>
       <c r="N28" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="O28" t="s">
         <v>291</v>

</xml_diff>

<commit_message>
working on benchtest head
</commit_message>
<xml_diff>
--- a/Doc/ConfigPrj/ExcelCfg/STM32G474RE/STM32G474RE_HwCfg.xlsx
+++ b/Doc/ConfigPrj/ExcelCfg/STM32G474RE/STM32G474RE_HwCfg.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\Software\STM32\Gamma_fMotionPlanner\Doc\ConfigPrj\ExcelCfg\STM32G474RE\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROJECT\STM32\ProjectGamma_Dev\Doc\ConfigPrj\ExcelCfg\STM32G474RE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0C2792E-3412-4261-8C95-67427E1660E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A9BA993-F2F3-4D36-ABF0-AF71ED517BE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2AF09063-600F-437A-B138-F66136E922A5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{2AF09063-600F-437A-B138-F66136E922A5}"/>
   </bookViews>
   <sheets>
     <sheet name="General_Info" sheetId="1" r:id="rId1"/>
@@ -2084,7 +2084,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="fr-FR"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -4833,7 +4833,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -5150,36 +5150,36 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{871E2D6D-43F7-44B1-8255-ECFDDA33AA9C}">
   <dimension ref="A17:AG119"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.6640625" customWidth="1"/>
-    <col min="2" max="2" width="24.77734375" customWidth="1"/>
-    <col min="3" max="3" width="37.33203125" customWidth="1"/>
-    <col min="4" max="4" width="26.44140625" customWidth="1"/>
-    <col min="5" max="6" width="25.109375" customWidth="1"/>
-    <col min="7" max="7" width="33.109375" customWidth="1"/>
-    <col min="8" max="8" width="26.88671875" customWidth="1"/>
-    <col min="9" max="9" width="21.44140625" customWidth="1"/>
-    <col min="10" max="10" width="21.33203125" customWidth="1"/>
-    <col min="12" max="12" width="20.44140625" customWidth="1"/>
-    <col min="13" max="13" width="29.44140625" customWidth="1"/>
-    <col min="14" max="14" width="21.33203125" customWidth="1"/>
-    <col min="15" max="15" width="22.77734375" customWidth="1"/>
-    <col min="16" max="16" width="23.44140625" customWidth="1"/>
-    <col min="17" max="17" width="20.6640625" customWidth="1"/>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="24.7109375" customWidth="1"/>
+    <col min="3" max="3" width="37.28515625" customWidth="1"/>
+    <col min="4" max="4" width="26.42578125" customWidth="1"/>
+    <col min="5" max="6" width="25.140625" customWidth="1"/>
+    <col min="7" max="7" width="33.140625" customWidth="1"/>
+    <col min="8" max="8" width="26.85546875" customWidth="1"/>
+    <col min="9" max="9" width="21.42578125" customWidth="1"/>
+    <col min="10" max="10" width="21.28515625" customWidth="1"/>
+    <col min="12" max="12" width="20.42578125" customWidth="1"/>
+    <col min="13" max="13" width="29.42578125" customWidth="1"/>
+    <col min="14" max="14" width="21.28515625" customWidth="1"/>
+    <col min="15" max="15" width="22.7109375" customWidth="1"/>
+    <col min="16" max="16" width="23.42578125" customWidth="1"/>
+    <col min="17" max="17" width="20.7109375" customWidth="1"/>
     <col min="18" max="18" width="21" customWidth="1"/>
-    <col min="19" max="19" width="33.88671875" customWidth="1"/>
-    <col min="20" max="20" width="35.33203125" customWidth="1"/>
-    <col min="21" max="21" width="21.21875" customWidth="1"/>
-    <col min="22" max="22" width="19.109375" customWidth="1"/>
-    <col min="23" max="23" width="18.77734375" customWidth="1"/>
-    <col min="24" max="24" width="29.21875" customWidth="1"/>
-    <col min="26" max="26" width="17.44140625" customWidth="1"/>
+    <col min="19" max="19" width="33.85546875" customWidth="1"/>
+    <col min="20" max="20" width="35.28515625" customWidth="1"/>
+    <col min="21" max="21" width="21.28515625" customWidth="1"/>
+    <col min="22" max="22" width="19.140625" customWidth="1"/>
+    <col min="23" max="23" width="18.7109375" customWidth="1"/>
+    <col min="24" max="24" width="29.28515625" customWidth="1"/>
+    <col min="26" max="26" width="17.42578125" customWidth="1"/>
     <col min="28" max="28" width="24" customWidth="1"/>
-    <col min="31" max="31" width="17.77734375" customWidth="1"/>
+    <col min="31" max="31" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="17" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:30" x14ac:dyDescent="0.25">
       <c r="R17" t="s">
         <v>452</v>
       </c>
@@ -5190,7 +5190,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="18" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:30" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
         <v>120</v>
       </c>
@@ -5234,7 +5234,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:30" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
         <v>121</v>
       </c>
@@ -5269,7 +5269,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="20" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:30" x14ac:dyDescent="0.25">
       <c r="D20" t="s">
         <v>228</v>
       </c>
@@ -5310,7 +5310,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="21" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:30" x14ac:dyDescent="0.25">
       <c r="D21" t="s">
         <v>231</v>
       </c>
@@ -5351,7 +5351,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="22" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:30" x14ac:dyDescent="0.25">
       <c r="D22" t="s">
         <v>232</v>
       </c>
@@ -5392,7 +5392,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="23" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:30" x14ac:dyDescent="0.25">
       <c r="D23" t="s">
         <v>233</v>
       </c>
@@ -5424,7 +5424,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="24" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:30" x14ac:dyDescent="0.25">
       <c r="D24" t="s">
         <v>234</v>
       </c>
@@ -5456,7 +5456,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="25" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:30" x14ac:dyDescent="0.25">
       <c r="D25" t="s">
         <v>82</v>
       </c>
@@ -5488,7 +5488,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="26" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:30" x14ac:dyDescent="0.25">
       <c r="D26" t="s">
         <v>257</v>
       </c>
@@ -5520,7 +5520,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="27" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>276</v>
       </c>
@@ -5558,7 +5558,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="28" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>277</v>
       </c>
@@ -5596,7 +5596,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="29" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>244</v>
       </c>
@@ -5634,7 +5634,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="30" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:30" x14ac:dyDescent="0.25">
       <c r="D30" t="s">
         <v>80</v>
       </c>
@@ -5666,7 +5666,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="31" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:30" x14ac:dyDescent="0.25">
       <c r="D31" t="s">
         <v>79</v>
       </c>
@@ -5683,7 +5683,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="32" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:30" x14ac:dyDescent="0.25">
       <c r="D32" t="s">
         <v>78</v>
       </c>
@@ -5700,7 +5700,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="33" spans="4:33" x14ac:dyDescent="0.3">
+    <row r="33" spans="4:33" x14ac:dyDescent="0.25">
       <c r="D33" t="s">
         <v>235</v>
       </c>
@@ -5723,7 +5723,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="34" spans="4:33" x14ac:dyDescent="0.3">
+    <row r="34" spans="4:33" x14ac:dyDescent="0.25">
       <c r="D34" t="s">
         <v>236</v>
       </c>
@@ -5746,7 +5746,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="35" spans="4:33" x14ac:dyDescent="0.3">
+    <row r="35" spans="4:33" x14ac:dyDescent="0.25">
       <c r="D35" t="s">
         <v>227</v>
       </c>
@@ -5769,7 +5769,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="36" spans="4:33" x14ac:dyDescent="0.3">
+    <row r="36" spans="4:33" x14ac:dyDescent="0.25">
       <c r="D36" t="s">
         <v>226</v>
       </c>
@@ -5798,7 +5798,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="37" spans="4:33" x14ac:dyDescent="0.3">
+    <row r="37" spans="4:33" x14ac:dyDescent="0.25">
       <c r="D37" t="s">
         <v>237</v>
       </c>
@@ -5827,7 +5827,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="38" spans="4:33" x14ac:dyDescent="0.3">
+    <row r="38" spans="4:33" x14ac:dyDescent="0.25">
       <c r="D38" t="s">
         <v>238</v>
       </c>
@@ -5850,7 +5850,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="39" spans="4:33" x14ac:dyDescent="0.3">
+    <row r="39" spans="4:33" x14ac:dyDescent="0.25">
       <c r="D39" t="s">
         <v>213</v>
       </c>
@@ -5873,7 +5873,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="40" spans="4:33" x14ac:dyDescent="0.3">
+    <row r="40" spans="4:33" x14ac:dyDescent="0.25">
       <c r="D40" t="s">
         <v>239</v>
       </c>
@@ -5914,7 +5914,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="41" spans="4:33" x14ac:dyDescent="0.3">
+    <row r="41" spans="4:33" x14ac:dyDescent="0.25">
       <c r="D41" t="s">
         <v>240</v>
       </c>
@@ -5946,7 +5946,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="42" spans="4:33" x14ac:dyDescent="0.3">
+    <row r="42" spans="4:33" x14ac:dyDescent="0.25">
       <c r="D42" t="s">
         <v>225</v>
       </c>
@@ -5978,7 +5978,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="43" spans="4:33" x14ac:dyDescent="0.3">
+    <row r="43" spans="4:33" x14ac:dyDescent="0.25">
       <c r="D43" t="s">
         <v>70</v>
       </c>
@@ -6010,7 +6010,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="44" spans="4:33" x14ac:dyDescent="0.3">
+    <row r="44" spans="4:33" x14ac:dyDescent="0.25">
       <c r="D44" t="s">
         <v>224</v>
       </c>
@@ -6039,7 +6039,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="45" spans="4:33" x14ac:dyDescent="0.3">
+    <row r="45" spans="4:33" x14ac:dyDescent="0.25">
       <c r="D45" t="s">
         <v>241</v>
       </c>
@@ -6068,7 +6068,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="46" spans="4:33" x14ac:dyDescent="0.3">
+    <row r="46" spans="4:33" x14ac:dyDescent="0.25">
       <c r="D46" t="s">
         <v>223</v>
       </c>
@@ -6088,7 +6088,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="47" spans="4:33" x14ac:dyDescent="0.3">
+    <row r="47" spans="4:33" x14ac:dyDescent="0.25">
       <c r="D47" t="s">
         <v>222</v>
       </c>
@@ -6108,7 +6108,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="48" spans="4:33" x14ac:dyDescent="0.3">
+    <row r="48" spans="4:33" x14ac:dyDescent="0.25">
       <c r="D48" t="s">
         <v>242</v>
       </c>
@@ -6128,7 +6128,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="49" spans="4:32" x14ac:dyDescent="0.3">
+    <row r="49" spans="4:32" x14ac:dyDescent="0.25">
       <c r="D49" t="s">
         <v>243</v>
       </c>
@@ -6148,7 +6148,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="50" spans="4:32" x14ac:dyDescent="0.3">
+    <row r="50" spans="4:32" x14ac:dyDescent="0.25">
       <c r="D50" t="s">
         <v>84</v>
       </c>
@@ -6165,7 +6165,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="51" spans="4:32" x14ac:dyDescent="0.3">
+    <row r="51" spans="4:32" x14ac:dyDescent="0.25">
       <c r="D51" t="s">
         <v>75</v>
       </c>
@@ -6182,7 +6182,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="52" spans="4:32" x14ac:dyDescent="0.3">
+    <row r="52" spans="4:32" x14ac:dyDescent="0.25">
       <c r="D52" t="s">
         <v>218</v>
       </c>
@@ -6202,7 +6202,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="53" spans="4:32" x14ac:dyDescent="0.3">
+    <row r="53" spans="4:32" x14ac:dyDescent="0.25">
       <c r="D53" t="s">
         <v>77</v>
       </c>
@@ -6222,7 +6222,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="54" spans="4:32" x14ac:dyDescent="0.3">
+    <row r="54" spans="4:32" x14ac:dyDescent="0.25">
       <c r="D54" t="s">
         <v>217</v>
       </c>
@@ -6242,7 +6242,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="55" spans="4:32" x14ac:dyDescent="0.3">
+    <row r="55" spans="4:32" x14ac:dyDescent="0.25">
       <c r="D55" t="s">
         <v>274</v>
       </c>
@@ -6262,7 +6262,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="56" spans="4:32" x14ac:dyDescent="0.3">
+    <row r="56" spans="4:32" x14ac:dyDescent="0.25">
       <c r="D56" t="s">
         <v>275</v>
       </c>
@@ -6282,7 +6282,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="57" spans="4:32" x14ac:dyDescent="0.3">
+    <row r="57" spans="4:32" x14ac:dyDescent="0.25">
       <c r="D57" t="s">
         <v>216</v>
       </c>
@@ -6302,7 +6302,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="58" spans="4:32" x14ac:dyDescent="0.3">
+    <row r="58" spans="4:32" x14ac:dyDescent="0.25">
       <c r="D58" t="s">
         <v>214</v>
       </c>
@@ -6322,7 +6322,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="59" spans="4:32" x14ac:dyDescent="0.3">
+    <row r="59" spans="4:32" x14ac:dyDescent="0.25">
       <c r="D59" t="s">
         <v>244</v>
       </c>
@@ -6342,7 +6342,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="60" spans="4:32" x14ac:dyDescent="0.3">
+    <row r="60" spans="4:32" x14ac:dyDescent="0.25">
       <c r="D60" t="s">
         <v>85</v>
       </c>
@@ -6362,7 +6362,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="61" spans="4:32" x14ac:dyDescent="0.3">
+    <row r="61" spans="4:32" x14ac:dyDescent="0.25">
       <c r="D61" t="s">
         <v>215</v>
       </c>
@@ -6382,7 +6382,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="62" spans="4:32" x14ac:dyDescent="0.3">
+    <row r="62" spans="4:32" x14ac:dyDescent="0.25">
       <c r="D62" t="s">
         <v>219</v>
       </c>
@@ -6402,7 +6402,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="63" spans="4:32" x14ac:dyDescent="0.3">
+    <row r="63" spans="4:32" x14ac:dyDescent="0.25">
       <c r="D63" t="s">
         <v>245</v>
       </c>
@@ -6419,7 +6419,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="64" spans="4:32" x14ac:dyDescent="0.3">
+    <row r="64" spans="4:32" x14ac:dyDescent="0.25">
       <c r="D64" t="s">
         <v>68</v>
       </c>
@@ -6436,7 +6436,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="65" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="65" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D65" t="s">
         <v>69</v>
       </c>
@@ -6453,7 +6453,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="66" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="66" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D66" t="s">
         <v>74</v>
       </c>
@@ -6470,7 +6470,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="67" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="67" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D67" t="s">
         <v>221</v>
       </c>
@@ -6487,7 +6487,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="68" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="68" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D68" t="s">
         <v>76</v>
       </c>
@@ -6504,7 +6504,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="69" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="69" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D69" t="s">
         <v>246</v>
       </c>
@@ -6521,7 +6521,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="70" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="70" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D70" t="s">
         <v>71</v>
       </c>
@@ -6538,7 +6538,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="71" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="71" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D71" t="s">
         <v>72</v>
       </c>
@@ -6555,7 +6555,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="72" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="72" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D72" t="s">
         <v>73</v>
       </c>
@@ -6572,7 +6572,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="73" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="73" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D73" t="s">
         <v>220</v>
       </c>
@@ -6589,7 +6589,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="74" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="74" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D74" t="s">
         <v>247</v>
       </c>
@@ -6606,7 +6606,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="75" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="75" spans="4:9" x14ac:dyDescent="0.25">
       <c r="D75" t="s">
         <v>248</v>
       </c>
@@ -6623,7 +6623,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="76" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="76" spans="4:9" x14ac:dyDescent="0.25">
       <c r="H76" t="s">
         <v>195</v>
       </c>
@@ -6631,7 +6631,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="77" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="77" spans="4:9" x14ac:dyDescent="0.25">
       <c r="H77" t="s">
         <v>194</v>
       </c>
@@ -6639,7 +6639,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="78" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="78" spans="4:9" x14ac:dyDescent="0.25">
       <c r="H78" t="s">
         <v>161</v>
       </c>
@@ -6647,7 +6647,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="79" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="79" spans="4:9" x14ac:dyDescent="0.25">
       <c r="H79" t="s">
         <v>202</v>
       </c>
@@ -6655,7 +6655,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="80" spans="4:9" x14ac:dyDescent="0.3">
+    <row r="80" spans="4:9" x14ac:dyDescent="0.25">
       <c r="H80" t="s">
         <v>122</v>
       </c>
@@ -6663,7 +6663,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="81" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="81" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H81" t="s">
         <v>206</v>
       </c>
@@ -6671,7 +6671,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="82" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="82" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H82" t="s">
         <v>59</v>
       </c>
@@ -6679,7 +6679,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="83" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="83" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H83" t="s">
         <v>201</v>
       </c>
@@ -6687,7 +6687,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="84" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="84" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H84" t="s">
         <v>153</v>
       </c>
@@ -6695,7 +6695,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="85" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="85" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H85" t="s">
         <v>123</v>
       </c>
@@ -6703,7 +6703,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="86" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="86" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H86" t="s">
         <v>124</v>
       </c>
@@ -6711,7 +6711,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="87" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="87" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H87" t="s">
         <v>188</v>
       </c>
@@ -6719,7 +6719,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="88" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="88" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H88" t="s">
         <v>63</v>
       </c>
@@ -6727,7 +6727,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="89" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="89" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H89" t="s">
         <v>64</v>
       </c>
@@ -6735,7 +6735,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="90" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="90" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H90" t="s">
         <v>163</v>
       </c>
@@ -6743,7 +6743,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="91" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="91" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H91" t="s">
         <v>196</v>
       </c>
@@ -6751,7 +6751,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="92" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="92" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H92" t="s">
         <v>142</v>
       </c>
@@ -6759,7 +6759,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="93" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="93" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H93" t="s">
         <v>61</v>
       </c>
@@ -6767,7 +6767,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="94" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="94" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H94" t="s">
         <v>144</v>
       </c>
@@ -6775,7 +6775,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="95" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="95" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H95" t="s">
         <v>143</v>
       </c>
@@ -6783,7 +6783,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="96" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="96" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H96" t="s">
         <v>145</v>
       </c>
@@ -6791,7 +6791,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="97" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="97" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H97" t="s">
         <v>189</v>
       </c>
@@ -6799,7 +6799,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="98" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="98" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H98" t="s">
         <v>192</v>
       </c>
@@ -6807,7 +6807,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="99" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="99" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H99" t="s">
         <v>191</v>
       </c>
@@ -6815,7 +6815,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="100" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="100" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H100" t="s">
         <v>190</v>
       </c>
@@ -6823,7 +6823,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="101" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="101" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H101" t="s">
         <v>62</v>
       </c>
@@ -6831,7 +6831,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="102" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="102" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H102" t="s">
         <v>146</v>
       </c>
@@ -6839,7 +6839,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="103" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="103" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H103" t="s">
         <v>162</v>
       </c>
@@ -6847,7 +6847,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="104" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="104" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H104" t="s">
         <v>166</v>
       </c>
@@ -6855,7 +6855,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="105" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="105" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H105" t="s">
         <v>167</v>
       </c>
@@ -6863,7 +6863,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="106" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="106" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H106" t="s">
         <v>155</v>
       </c>
@@ -6871,7 +6871,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="107" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="107" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H107" t="s">
         <v>158</v>
       </c>
@@ -6879,7 +6879,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="108" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="108" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H108" t="s">
         <v>157</v>
       </c>
@@ -6887,7 +6887,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="109" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="109" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H109" t="s">
         <v>156</v>
       </c>
@@ -6895,7 +6895,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="110" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="110" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H110" t="s">
         <v>164</v>
       </c>
@@ -6903,7 +6903,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="111" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="111" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H111" t="s">
         <v>165</v>
       </c>
@@ -6911,7 +6911,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="112" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="112" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H112" t="s">
         <v>175</v>
       </c>
@@ -6919,7 +6919,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="113" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="113" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H113" t="s">
         <v>65</v>
       </c>
@@ -6927,7 +6927,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="114" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="114" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H114" t="s">
         <v>66</v>
       </c>
@@ -6935,7 +6935,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="115" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="115" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H115" t="s">
         <v>151</v>
       </c>
@@ -6943,7 +6943,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="116" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="116" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H116" t="s">
         <v>137</v>
       </c>
@@ -6951,7 +6951,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="117" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="117" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H117" t="s">
         <v>138</v>
       </c>
@@ -6959,7 +6959,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="118" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="118" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H118" t="s">
         <v>154</v>
       </c>
@@ -6967,7 +6967,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="119" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="119" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H119" t="s">
         <v>57</v>
       </c>
@@ -7014,18 +7014,18 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34ECC9F7-B649-41BF-A742-3CCEA0266A56}">
   <dimension ref="B3:R28"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="5" max="5" width="18.77734375" customWidth="1"/>
-    <col min="6" max="6" width="20.77734375" customWidth="1"/>
+    <col min="5" max="5" width="18.7109375" customWidth="1"/>
+    <col min="6" max="6" width="20.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:15" ht="93.6" x14ac:dyDescent="1.75">
+    <row r="3" spans="2:15" ht="93.75" x14ac:dyDescent="1.4">
       <c r="B3" s="6" t="s">
         <v>430</v>
       </c>
     </row>
-    <row r="5" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:15" x14ac:dyDescent="0.25">
       <c r="J5" t="s">
         <v>442</v>
       </c>
@@ -7036,7 +7036,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="6" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:15" x14ac:dyDescent="0.25">
       <c r="J6">
         <v>128000000</v>
       </c>
@@ -7047,47 +7047,47 @@
         <v>64000</v>
       </c>
     </row>
-    <row r="8" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:15" x14ac:dyDescent="0.25">
       <c r="O8">
         <v>32</v>
       </c>
     </row>
-    <row r="9" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:15" x14ac:dyDescent="0.25">
       <c r="O9">
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:15" x14ac:dyDescent="0.25">
       <c r="O10">
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:15" x14ac:dyDescent="0.25">
       <c r="O11">
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:15" x14ac:dyDescent="0.25">
       <c r="O12">
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:15" x14ac:dyDescent="0.25">
       <c r="O13">
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:15" x14ac:dyDescent="0.25">
       <c r="O14">
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:15" x14ac:dyDescent="0.25">
       <c r="O15">
         <v>4</v>
       </c>
     </row>
-    <row r="20" spans="5:18" x14ac:dyDescent="0.3">
+    <row r="20" spans="5:18" x14ac:dyDescent="0.25">
       <c r="E20" s="9" t="s">
         <v>439</v>
       </c>
@@ -7098,7 +7098,7 @@
         <v>440</v>
       </c>
     </row>
-    <row r="21" spans="5:18" x14ac:dyDescent="0.3">
+    <row r="21" spans="5:18" x14ac:dyDescent="0.25">
       <c r="E21" s="7" t="s">
         <v>431</v>
       </c>
@@ -7111,7 +7111,7 @@
         <v>64000</v>
       </c>
     </row>
-    <row r="22" spans="5:18" x14ac:dyDescent="0.3">
+    <row r="22" spans="5:18" x14ac:dyDescent="0.25">
       <c r="E22" s="8" t="s">
         <v>432</v>
       </c>
@@ -7124,7 +7124,7 @@
         <v>32000</v>
       </c>
     </row>
-    <row r="23" spans="5:18" x14ac:dyDescent="0.3">
+    <row r="23" spans="5:18" x14ac:dyDescent="0.25">
       <c r="E23" s="7" t="s">
         <v>433</v>
       </c>
@@ -7140,7 +7140,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="24" spans="5:18" x14ac:dyDescent="0.3">
+    <row r="24" spans="5:18" x14ac:dyDescent="0.25">
       <c r="E24" s="8" t="s">
         <v>434</v>
       </c>
@@ -7153,7 +7153,7 @@
         <v>8000</v>
       </c>
     </row>
-    <row r="25" spans="5:18" x14ac:dyDescent="0.3">
+    <row r="25" spans="5:18" x14ac:dyDescent="0.25">
       <c r="E25" s="7" t="s">
         <v>435</v>
       </c>
@@ -7166,7 +7166,7 @@
         <v>4000</v>
       </c>
     </row>
-    <row r="26" spans="5:18" x14ac:dyDescent="0.3">
+    <row r="26" spans="5:18" x14ac:dyDescent="0.25">
       <c r="E26" s="8" t="s">
         <v>436</v>
       </c>
@@ -7179,7 +7179,7 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="27" spans="5:18" x14ac:dyDescent="0.3">
+    <row r="27" spans="5:18" x14ac:dyDescent="0.25">
       <c r="E27" s="7" t="s">
         <v>437</v>
       </c>
@@ -7192,7 +7192,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="28" spans="5:18" x14ac:dyDescent="0.3">
+    <row r="28" spans="5:18" x14ac:dyDescent="0.25">
       <c r="E28" s="11" t="s">
         <v>438</v>
       </c>
@@ -7216,39 +7216,39 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{492C7761-01BE-400F-9C40-BE71D85F5C61}">
   <dimension ref="A2:BA57"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.109375" customWidth="1"/>
-    <col min="2" max="2" width="24.77734375" customWidth="1"/>
-    <col min="3" max="3" width="25.33203125" customWidth="1"/>
+    <col min="1" max="1" width="25.140625" customWidth="1"/>
+    <col min="2" max="2" width="24.7109375" customWidth="1"/>
+    <col min="3" max="3" width="25.28515625" customWidth="1"/>
     <col min="5" max="5" width="25" customWidth="1"/>
-    <col min="6" max="6" width="22.109375" customWidth="1"/>
+    <col min="6" max="6" width="22.140625" customWidth="1"/>
     <col min="7" max="7" width="25" customWidth="1"/>
-    <col min="8" max="8" width="22.88671875" customWidth="1"/>
-    <col min="9" max="9" width="15.21875" customWidth="1"/>
-    <col min="10" max="10" width="24.109375" customWidth="1"/>
-    <col min="12" max="12" width="21.109375" customWidth="1"/>
-    <col min="13" max="13" width="17.5546875" customWidth="1"/>
-    <col min="14" max="14" width="18.109375" customWidth="1"/>
-    <col min="15" max="15" width="28.5546875" customWidth="1"/>
-    <col min="16" max="16" width="24.6640625" customWidth="1"/>
-    <col min="18" max="18" width="18.5546875" customWidth="1"/>
-    <col min="19" max="19" width="23.33203125" customWidth="1"/>
-    <col min="20" max="20" width="18.44140625" customWidth="1"/>
-    <col min="21" max="21" width="23.109375" customWidth="1"/>
-    <col min="23" max="23" width="25.109375" customWidth="1"/>
+    <col min="8" max="8" width="22.85546875" customWidth="1"/>
+    <col min="9" max="9" width="15.28515625" customWidth="1"/>
+    <col min="10" max="10" width="24.140625" customWidth="1"/>
+    <col min="12" max="12" width="21.140625" customWidth="1"/>
+    <col min="13" max="13" width="17.5703125" customWidth="1"/>
+    <col min="14" max="14" width="18.140625" customWidth="1"/>
+    <col min="15" max="15" width="28.5703125" customWidth="1"/>
+    <col min="16" max="16" width="24.7109375" customWidth="1"/>
+    <col min="18" max="18" width="18.5703125" customWidth="1"/>
+    <col min="19" max="19" width="23.28515625" customWidth="1"/>
+    <col min="20" max="20" width="18.42578125" customWidth="1"/>
+    <col min="21" max="21" width="23.140625" customWidth="1"/>
+    <col min="23" max="23" width="25.140625" customWidth="1"/>
     <col min="24" max="24" width="34" customWidth="1"/>
-    <col min="25" max="25" width="16.77734375" customWidth="1"/>
-    <col min="26" max="26" width="20.77734375" customWidth="1"/>
-    <col min="27" max="27" width="16.77734375" customWidth="1"/>
+    <col min="25" max="25" width="16.7109375" customWidth="1"/>
+    <col min="26" max="26" width="20.7109375" customWidth="1"/>
+    <col min="27" max="27" width="16.7109375" customWidth="1"/>
     <col min="30" max="30" width="13" customWidth="1"/>
-    <col min="31" max="31" width="17.6640625" customWidth="1"/>
-    <col min="38" max="38" width="17.21875" customWidth="1"/>
-    <col min="40" max="40" width="19.44140625" customWidth="1"/>
-    <col min="53" max="53" width="40.5546875" customWidth="1"/>
+    <col min="31" max="31" width="17.7109375" customWidth="1"/>
+    <col min="38" max="38" width="17.28515625" customWidth="1"/>
+    <col min="40" max="40" width="19.42578125" customWidth="1"/>
+    <col min="53" max="53" width="40.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>429</v>
       </c>
@@ -7256,7 +7256,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>51</v>
       </c>
@@ -7279,7 +7279,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -7344,7 +7344,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -7412,7 +7412,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -7480,7 +7480,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" x14ac:dyDescent="0.25">
       <c r="E9" t="s">
         <v>10</v>
       </c>
@@ -7494,10 +7494,10 @@
         <v>104</v>
       </c>
       <c r="J9" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="K9" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="L9" t="s">
         <v>425</v>
@@ -7542,7 +7542,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.25">
       <c r="E10" t="s">
         <v>10</v>
       </c>
@@ -7556,10 +7556,10 @@
         <v>107</v>
       </c>
       <c r="J10" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="K10" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="L10" t="s">
         <v>425</v>
@@ -7604,7 +7604,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" x14ac:dyDescent="0.25">
       <c r="E11" t="s">
         <v>9</v>
       </c>
@@ -7645,13 +7645,13 @@
         <v>500</v>
       </c>
       <c r="AA11" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AB11" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.3">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
       <c r="P12" t="s">
         <v>9</v>
       </c>
@@ -7680,13 +7680,13 @@
         <v>427</v>
       </c>
       <c r="AA12" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="AB12" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.3">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="13" spans="1:28" x14ac:dyDescent="0.25">
       <c r="P13" t="s">
         <v>11</v>
       </c>
@@ -7718,10 +7718,10 @@
         <v>13</v>
       </c>
       <c r="AB13" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.3">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14" spans="1:28" x14ac:dyDescent="0.25">
       <c r="P14" s="13" t="s">
         <v>9</v>
       </c>
@@ -7750,13 +7750,13 @@
         <v>500</v>
       </c>
       <c r="AA14" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="AB14" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.3">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="15" spans="1:28" x14ac:dyDescent="0.25">
       <c r="P15" s="15" t="s">
         <v>9</v>
       </c>
@@ -7776,13 +7776,13 @@
         <v>456</v>
       </c>
       <c r="AA15" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="AB15" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:28" x14ac:dyDescent="0.25">
       <c r="P16" s="13" t="s">
         <v>10</v>
       </c>
@@ -7802,7 +7802,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="17" spans="16:53" x14ac:dyDescent="0.3">
+    <row r="17" spans="16:53" x14ac:dyDescent="0.25">
       <c r="P17" s="15" t="s">
         <v>10</v>
       </c>
@@ -7822,7 +7822,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="18" spans="16:53" x14ac:dyDescent="0.3">
+    <row r="18" spans="16:53" x14ac:dyDescent="0.25">
       <c r="P18" s="13" t="s">
         <v>11</v>
       </c>
@@ -7842,7 +7842,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="19" spans="16:53" x14ac:dyDescent="0.3">
+    <row r="19" spans="16:53" x14ac:dyDescent="0.25">
       <c r="P19" s="15" t="s">
         <v>11</v>
       </c>
@@ -7862,7 +7862,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="20" spans="16:53" x14ac:dyDescent="0.3">
+    <row r="20" spans="16:53" x14ac:dyDescent="0.25">
       <c r="P20" t="s">
         <v>11</v>
       </c>
@@ -7882,17 +7882,17 @@
         <v>456</v>
       </c>
     </row>
-    <row r="27" spans="16:53" x14ac:dyDescent="0.3">
+    <row r="27" spans="16:53" x14ac:dyDescent="0.25">
       <c r="W27" t="s">
         <v>354</v>
       </c>
     </row>
-    <row r="28" spans="16:53" x14ac:dyDescent="0.3">
+    <row r="28" spans="16:53" x14ac:dyDescent="0.25">
       <c r="W28" t="s">
         <v>347</v>
       </c>
     </row>
-    <row r="29" spans="16:53" x14ac:dyDescent="0.3">
+    <row r="29" spans="16:53" x14ac:dyDescent="0.25">
       <c r="W29" t="s">
         <v>355</v>
       </c>
@@ -7903,7 +7903,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="30" spans="16:53" x14ac:dyDescent="0.3">
+    <row r="30" spans="16:53" x14ac:dyDescent="0.25">
       <c r="W30" t="s">
         <v>356</v>
       </c>
@@ -7917,7 +7917,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="31" spans="16:53" x14ac:dyDescent="0.3">
+    <row r="31" spans="16:53" x14ac:dyDescent="0.25">
       <c r="W31" t="s">
         <v>357</v>
       </c>
@@ -7931,7 +7931,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="32" spans="16:53" x14ac:dyDescent="0.3">
+    <row r="32" spans="16:53" x14ac:dyDescent="0.25">
       <c r="W32" t="s">
         <v>358</v>
       </c>
@@ -7945,7 +7945,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="33" spans="2:53" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:53" x14ac:dyDescent="0.25">
       <c r="W33" t="s">
         <v>359</v>
       </c>
@@ -7959,7 +7959,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="34" spans="2:53" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:53" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
         <v>403</v>
       </c>
@@ -7976,7 +7976,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="35" spans="2:53" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:53" x14ac:dyDescent="0.25">
       <c r="B35" t="s">
         <v>281</v>
       </c>
@@ -8005,7 +8005,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="36" spans="2:53" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:53" x14ac:dyDescent="0.25">
       <c r="B36" t="s">
         <v>13</v>
       </c>
@@ -8031,7 +8031,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="37" spans="2:53" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:53" x14ac:dyDescent="0.25">
       <c r="B37" t="s">
         <v>256</v>
       </c>
@@ -8057,7 +8057,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="38" spans="2:53" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:53" x14ac:dyDescent="0.25">
       <c r="B38" t="s">
         <v>256</v>
       </c>
@@ -8083,7 +8083,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="39" spans="2:53" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:53" x14ac:dyDescent="0.25">
       <c r="AW39" t="s">
         <v>32</v>
       </c>
@@ -8091,7 +8091,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="40" spans="2:53" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:53" x14ac:dyDescent="0.25">
       <c r="AW40" t="s">
         <v>33</v>
       </c>
@@ -8099,7 +8099,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="41" spans="2:53" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:53" x14ac:dyDescent="0.25">
       <c r="AW41" t="s">
         <v>34</v>
       </c>
@@ -8107,7 +8107,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="42" spans="2:53" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:53" x14ac:dyDescent="0.25">
       <c r="AW42" t="s">
         <v>36</v>
       </c>
@@ -8115,7 +8115,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="43" spans="2:53" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:53" x14ac:dyDescent="0.25">
       <c r="AW43" t="s">
         <v>37</v>
       </c>
@@ -8123,7 +8123,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="44" spans="2:53" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:53" x14ac:dyDescent="0.25">
       <c r="B44" s="9" t="s">
         <v>491</v>
       </c>
@@ -8152,7 +8152,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="45" spans="2:53" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:53" x14ac:dyDescent="0.25">
       <c r="B45" s="16"/>
       <c r="C45" s="16"/>
       <c r="D45" s="16"/>
@@ -8167,22 +8167,22 @@
         <v>107</v>
       </c>
     </row>
-    <row r="46" spans="2:53" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:53" x14ac:dyDescent="0.25">
       <c r="BA46" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="47" spans="2:53" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:53" x14ac:dyDescent="0.25">
       <c r="BA47" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="48" spans="2:53" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:53" x14ac:dyDescent="0.25">
       <c r="BA48" t="s">
         <v>472</v>
       </c>
     </row>
-    <row r="57" spans="36:36" x14ac:dyDescent="0.3">
+    <row r="57" spans="36:36" x14ac:dyDescent="0.25">
       <c r="AJ57" t="s">
         <v>110</v>
       </c>
@@ -8190,7 +8190,7 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <dataValidations count="5">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AW46 Q14:Q19 Q7 K7:K10 AB8:AB13 F7:F10 F11 X7:X14 AB15 B7:B8" xr:uid="{14BC2D73-1395-4E2C-9D1E-55C781825C64}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AW46 Q14:Q19 Q7 AB8:AB12 F7:F11 X7:X14 AB14 B7:B8 K7:K10" xr:uid="{14BC2D73-1395-4E2C-9D1E-55C781825C64}">
       <formula1>$AW$30:$AW$45</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="T14:T19 T7 N7:N10" xr:uid="{727A5344-B28A-4866-9EC1-7C96029AF8B6}">
@@ -8229,7 +8229,7 @@
           <x14:formula1>
             <xm:f>General_Info!$P$34:$P$39</xm:f>
           </x14:formula1>
-          <xm:sqref>P14:P19 P7 J7:J10 AA8:AA13 E7:E10 E11 W7:W14 AA15 A7:A8</xm:sqref>
+          <xm:sqref>P14:P19 P7 AA8:AA12 E7:E11 W7:W14 AA14 A7:A8 J7:J10</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{3C428027-B16D-4B04-9CB2-8290577ED0FB}">
           <x14:formula1>
@@ -8246,15 +8246,15 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1E52BA6-3E0A-4F7C-9391-164B38476F25}">
   <dimension ref="B3:G17"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="19.44140625" customWidth="1"/>
-    <col min="3" max="3" width="22.21875" customWidth="1"/>
-    <col min="6" max="6" width="31.33203125" customWidth="1"/>
-    <col min="7" max="7" width="26.6640625" customWidth="1"/>
+    <col min="2" max="2" width="19.42578125" customWidth="1"/>
+    <col min="3" max="3" width="22.28515625" customWidth="1"/>
+    <col min="6" max="6" width="31.28515625" customWidth="1"/>
+    <col min="7" max="7" width="26.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>49</v>
       </c>
@@ -8262,7 +8262,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="4" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>0</v>
       </c>
@@ -8276,7 +8276,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="5" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>250</v>
       </c>
@@ -8290,7 +8290,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="6" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>251</v>
       </c>
@@ -8304,7 +8304,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="7" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
       <c r="F7" t="s">
         <v>343</v>
       </c>
@@ -8312,7 +8312,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="8" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
       <c r="F8" t="s">
         <v>342</v>
       </c>
@@ -8320,7 +8320,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="9" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
       <c r="F9" t="s">
         <v>344</v>
       </c>
@@ -8328,7 +8328,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="10" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:7" x14ac:dyDescent="0.25">
       <c r="F10" t="s">
         <v>345</v>
       </c>
@@ -8336,7 +8336,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="11" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:7" x14ac:dyDescent="0.25">
       <c r="F11" t="s">
         <v>346</v>
       </c>
@@ -8344,7 +8344,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="12" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:7" x14ac:dyDescent="0.25">
       <c r="F12" t="s">
         <v>348</v>
       </c>
@@ -8352,7 +8352,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="13" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:7" x14ac:dyDescent="0.25">
       <c r="F13" t="s">
         <v>349</v>
       </c>
@@ -8360,7 +8360,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="14" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:7" x14ac:dyDescent="0.25">
       <c r="F14" t="s">
         <v>426</v>
       </c>
@@ -8368,7 +8368,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="15" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:7" x14ac:dyDescent="0.25">
       <c r="F15" t="s">
         <v>350</v>
       </c>
@@ -8376,7 +8376,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="16" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:7" x14ac:dyDescent="0.25">
       <c r="F16" t="s">
         <v>351</v>
       </c>
@@ -8384,7 +8384,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="17" spans="6:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="6:7" x14ac:dyDescent="0.25">
       <c r="F17" t="s">
         <v>353</v>
       </c>
@@ -8405,47 +8405,47 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7BF150CB-3330-4180-96AC-4A3D28CDB7F6}">
   <dimension ref="Y5:Y12"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="25" max="25" width="27.21875" customWidth="1"/>
+    <col min="25" max="25" width="27.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="5" spans="25:25" x14ac:dyDescent="0.3">
+    <row r="5" spans="25:25" x14ac:dyDescent="0.25">
       <c r="Y5" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="25:25" x14ac:dyDescent="0.3">
+    <row r="6" spans="25:25" x14ac:dyDescent="0.25">
       <c r="Y6" t="s">
         <v>447</v>
       </c>
     </row>
-    <row r="7" spans="25:25" x14ac:dyDescent="0.3">
+    <row r="7" spans="25:25" x14ac:dyDescent="0.25">
       <c r="Y7" t="s">
         <v>446</v>
       </c>
     </row>
-    <row r="8" spans="25:25" x14ac:dyDescent="0.3">
+    <row r="8" spans="25:25" x14ac:dyDescent="0.25">
       <c r="Y8" t="s">
         <v>448</v>
       </c>
     </row>
-    <row r="9" spans="25:25" x14ac:dyDescent="0.3">
+    <row r="9" spans="25:25" x14ac:dyDescent="0.25">
       <c r="Y9" t="s">
         <v>445</v>
       </c>
     </row>
-    <row r="10" spans="25:25" x14ac:dyDescent="0.3">
+    <row r="10" spans="25:25" x14ac:dyDescent="0.25">
       <c r="Y10" t="s">
         <v>449</v>
       </c>
     </row>
-    <row r="11" spans="25:25" x14ac:dyDescent="0.3">
+    <row r="11" spans="25:25" x14ac:dyDescent="0.25">
       <c r="Y11" t="s">
         <v>450</v>
       </c>
     </row>
-    <row r="12" spans="25:25" x14ac:dyDescent="0.3">
+    <row r="12" spans="25:25" x14ac:dyDescent="0.25">
       <c r="Y12" t="s">
         <v>451</v>
       </c>
@@ -8461,22 +8461,22 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0962FBCC-E1F3-44E3-92A8-D1FF17927B08}">
   <dimension ref="E2:W22"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="5" max="5" width="23.44140625" customWidth="1"/>
-    <col min="6" max="6" width="22.44140625" customWidth="1"/>
-    <col min="9" max="9" width="43.88671875" customWidth="1"/>
-    <col min="10" max="10" width="21.6640625" customWidth="1"/>
-    <col min="11" max="11" width="11.5546875" customWidth="1"/>
-    <col min="12" max="12" width="24.109375" customWidth="1"/>
+    <col min="5" max="5" width="23.42578125" customWidth="1"/>
+    <col min="6" max="6" width="22.42578125" customWidth="1"/>
+    <col min="9" max="9" width="43.85546875" customWidth="1"/>
+    <col min="10" max="10" width="21.7109375" customWidth="1"/>
+    <col min="11" max="11" width="11.5703125" customWidth="1"/>
+    <col min="12" max="12" width="24.140625" customWidth="1"/>
     <col min="17" max="17" width="45" customWidth="1"/>
-    <col min="18" max="18" width="28.88671875" customWidth="1"/>
-    <col min="19" max="19" width="21.88671875" customWidth="1"/>
-    <col min="20" max="20" width="19.21875" customWidth="1"/>
-    <col min="22" max="22" width="18.5546875" customWidth="1"/>
+    <col min="18" max="18" width="28.85546875" customWidth="1"/>
+    <col min="19" max="19" width="21.85546875" customWidth="1"/>
+    <col min="20" max="20" width="19.28515625" customWidth="1"/>
+    <col min="22" max="22" width="18.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="5:17" ht="25.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="5:17" ht="25.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I2" s="3" t="s">
         <v>115</v>
       </c>
@@ -8484,7 +8484,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="3" spans="5:17" x14ac:dyDescent="0.3">
+    <row r="3" spans="5:17" x14ac:dyDescent="0.25">
       <c r="I3" t="s">
         <v>112</v>
       </c>
@@ -8501,7 +8501,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="4" spans="5:17" x14ac:dyDescent="0.3">
+    <row r="4" spans="5:17" x14ac:dyDescent="0.25">
       <c r="I4" t="s">
         <v>474</v>
       </c>
@@ -8518,7 +8518,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="5" spans="5:17" x14ac:dyDescent="0.3">
+    <row r="5" spans="5:17" x14ac:dyDescent="0.25">
       <c r="I5" t="s">
         <v>111</v>
       </c>
@@ -8535,7 +8535,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="6" spans="5:17" x14ac:dyDescent="0.3">
+    <row r="6" spans="5:17" x14ac:dyDescent="0.25">
       <c r="I6" t="s">
         <v>262</v>
       </c>
@@ -8552,12 +8552,12 @@
         <v>478</v>
       </c>
     </row>
-    <row r="7" spans="5:17" x14ac:dyDescent="0.3">
+    <row r="7" spans="5:17" x14ac:dyDescent="0.25">
       <c r="E7" t="s">
         <v>354</v>
       </c>
     </row>
-    <row r="8" spans="5:17" x14ac:dyDescent="0.3">
+    <row r="8" spans="5:17" x14ac:dyDescent="0.25">
       <c r="E8" t="s">
         <v>347</v>
       </c>
@@ -8565,7 +8565,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="9" spans="5:17" x14ac:dyDescent="0.3">
+    <row r="9" spans="5:17" x14ac:dyDescent="0.25">
       <c r="E9" t="s">
         <v>362</v>
       </c>
@@ -8573,7 +8573,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="10" spans="5:17" x14ac:dyDescent="0.3">
+    <row r="10" spans="5:17" x14ac:dyDescent="0.25">
       <c r="E10" t="s">
         <v>363</v>
       </c>
@@ -8581,7 +8581,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="11" spans="5:17" x14ac:dyDescent="0.3">
+    <row r="11" spans="5:17" x14ac:dyDescent="0.25">
       <c r="E11" t="s">
         <v>364</v>
       </c>
@@ -8589,7 +8589,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="12" spans="5:17" x14ac:dyDescent="0.3">
+    <row r="12" spans="5:17" x14ac:dyDescent="0.25">
       <c r="E12" t="s">
         <v>365</v>
       </c>
@@ -8597,7 +8597,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="17" spans="20:23" x14ac:dyDescent="0.3">
+    <row r="17" spans="20:23" x14ac:dyDescent="0.25">
       <c r="T17" t="s">
         <v>114</v>
       </c>
@@ -8611,7 +8611,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="18" spans="20:23" x14ac:dyDescent="0.3">
+    <row r="18" spans="20:23" x14ac:dyDescent="0.25">
       <c r="T18" t="s">
         <v>413</v>
       </c>
@@ -8625,7 +8625,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="19" spans="20:23" x14ac:dyDescent="0.3">
+    <row r="19" spans="20:23" x14ac:dyDescent="0.25">
       <c r="T19" t="s">
         <v>414</v>
       </c>
@@ -8639,7 +8639,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="20" spans="20:23" x14ac:dyDescent="0.3">
+    <row r="20" spans="20:23" x14ac:dyDescent="0.25">
       <c r="T20" t="s">
         <v>415</v>
       </c>
@@ -8653,7 +8653,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="21" spans="20:23" x14ac:dyDescent="0.3">
+    <row r="21" spans="20:23" x14ac:dyDescent="0.25">
       <c r="T21" t="s">
         <v>416</v>
       </c>
@@ -8667,7 +8667,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="22" spans="20:23" x14ac:dyDescent="0.3">
+    <row r="22" spans="20:23" x14ac:dyDescent="0.25">
       <c r="T22" t="s">
         <v>417</v>
       </c>
@@ -8713,22 +8713,22 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06E18236-E25D-41B3-8B1E-0194276152B3}">
   <dimension ref="B1:P18"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="19.33203125" customWidth="1"/>
-    <col min="3" max="3" width="17.77734375" customWidth="1"/>
-    <col min="4" max="4" width="17.44140625" customWidth="1"/>
-    <col min="10" max="10" width="36.6640625" customWidth="1"/>
-    <col min="11" max="11" width="21.77734375" customWidth="1"/>
-    <col min="16" max="16" width="25.33203125" customWidth="1"/>
+    <col min="2" max="2" width="19.28515625" customWidth="1"/>
+    <col min="3" max="3" width="17.7109375" customWidth="1"/>
+    <col min="4" max="4" width="17.42578125" customWidth="1"/>
+    <col min="10" max="10" width="36.7109375" customWidth="1"/>
+    <col min="11" max="11" width="21.7109375" customWidth="1"/>
+    <col min="16" max="16" width="25.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
         <v>489</v>
       </c>
     </row>
-    <row r="2" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>329</v>
       </c>
@@ -8745,7 +8745,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="3" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>326</v>
       </c>
@@ -8768,7 +8768,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="4" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>401</v>
       </c>
@@ -8794,7 +8794,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="5" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>391</v>
       </c>
@@ -8814,7 +8814,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="6" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>392</v>
       </c>
@@ -8834,7 +8834,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="7" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>393</v>
       </c>
@@ -8854,7 +8854,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="8" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>334</v>
       </c>
@@ -8874,7 +8874,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="9" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>335</v>
       </c>
@@ -8894,12 +8894,12 @@
         <v>336</v>
       </c>
     </row>
-    <row r="10" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>336</v>
       </c>
       <c r="C10" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="D10" t="s">
         <v>337</v>
@@ -8914,12 +8914,12 @@
         <v>338</v>
       </c>
     </row>
-    <row r="11" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>338</v>
       </c>
       <c r="C11" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="D11" t="s">
         <v>339</v>
@@ -8934,7 +8934,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="12" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>397</v>
       </c>
@@ -8954,7 +8954,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="13" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>398</v>
       </c>
@@ -8974,12 +8974,12 @@
         <v>422</v>
       </c>
     </row>
-    <row r="14" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>487</v>
       </c>
       <c r="C14" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D14" t="s">
         <v>337</v>
@@ -8994,12 +8994,12 @@
         <v>487</v>
       </c>
     </row>
-    <row r="15" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>488</v>
       </c>
       <c r="C15" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D15" t="s">
         <v>339</v>
@@ -9014,7 +9014,7 @@
         <v>488</v>
       </c>
     </row>
-    <row r="16" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
         <v>422</v>
       </c>
@@ -9031,12 +9031,12 @@
         <v>378</v>
       </c>
     </row>
-    <row r="17" spans="10:10" x14ac:dyDescent="0.3">
+    <row r="17" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J17" t="s">
         <v>379</v>
       </c>
     </row>
-    <row r="18" spans="10:10" x14ac:dyDescent="0.3">
+    <row r="18" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J18" t="s">
         <v>380</v>
       </c>
@@ -9054,23 +9054,23 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9D1D4C8-FD0D-4DBE-B311-5297C41CC83F}">
   <dimension ref="A1:G11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="23.77734375" customWidth="1"/>
+    <col min="2" max="2" width="23.7109375" customWidth="1"/>
     <col min="6" max="6" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>381</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>354</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>347</v>
       </c>
@@ -9087,7 +9087,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>382</v>
       </c>
@@ -9104,7 +9104,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>383</v>
       </c>
@@ -9121,7 +9121,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>384</v>
       </c>
@@ -9138,17 +9138,17 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>385</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>386</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>387</v>
       </c>
@@ -9166,21 +9166,21 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E85D06B3-E762-495B-BF06-A6CD7E704A4C}">
   <dimension ref="E2:M7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="15.6640625" customWidth="1"/>
+    <col min="2" max="2" width="15.7109375" customWidth="1"/>
     <col min="5" max="5" width="17" customWidth="1"/>
-    <col min="6" max="6" width="19.6640625" customWidth="1"/>
-    <col min="7" max="7" width="15.33203125" customWidth="1"/>
-    <col min="8" max="8" width="16.109375" customWidth="1"/>
-    <col min="9" max="9" width="18.44140625" customWidth="1"/>
-    <col min="10" max="10" width="20.44140625" customWidth="1"/>
-    <col min="11" max="11" width="23.33203125" customWidth="1"/>
-    <col min="12" max="12" width="18.6640625" customWidth="1"/>
-    <col min="13" max="13" width="19.6640625" customWidth="1"/>
+    <col min="6" max="6" width="19.7109375" customWidth="1"/>
+    <col min="7" max="7" width="15.28515625" customWidth="1"/>
+    <col min="8" max="8" width="16.140625" customWidth="1"/>
+    <col min="9" max="9" width="18.42578125" customWidth="1"/>
+    <col min="10" max="10" width="20.42578125" customWidth="1"/>
+    <col min="11" max="11" width="23.28515625" customWidth="1"/>
+    <col min="12" max="12" width="18.7109375" customWidth="1"/>
+    <col min="13" max="13" width="19.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="5:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="5:13" x14ac:dyDescent="0.25">
       <c r="E2" t="s">
         <v>405</v>
       </c>
@@ -9209,7 +9209,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="5:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="5:13" x14ac:dyDescent="0.25">
       <c r="E3" t="s">
         <v>76</v>
       </c>
@@ -9238,7 +9238,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="4" spans="5:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="5:13" x14ac:dyDescent="0.25">
       <c r="E4" t="s">
         <v>77</v>
       </c>
@@ -9267,7 +9267,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="5" spans="5:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="5:13" x14ac:dyDescent="0.25">
       <c r="E5" t="s">
         <v>217</v>
       </c>
@@ -9275,28 +9275,28 @@
         <v>408</v>
       </c>
       <c r="G5">
-        <v>0</v>
+        <v>256</v>
       </c>
       <c r="H5">
-        <v>0</v>
+        <v>2048</v>
       </c>
       <c r="I5" t="s">
-        <v>256</v>
+        <v>10</v>
       </c>
       <c r="J5" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="K5" t="s">
-        <v>256</v>
+        <v>10</v>
       </c>
       <c r="L5" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="M5" t="s">
         <v>419</v>
       </c>
     </row>
-    <row r="6" spans="5:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="5:13" x14ac:dyDescent="0.25">
       <c r="E6" t="s">
         <v>274</v>
       </c>
@@ -9325,7 +9325,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="7" spans="5:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="5:13" x14ac:dyDescent="0.25">
       <c r="E7" t="s">
         <v>275</v>
       </c>
@@ -9366,27 +9366,27 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{860CCB6B-9BC8-4B28-B4AE-B22F38F81573}">
   <dimension ref="B1:P254"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="17.5546875" customWidth="1"/>
-    <col min="5" max="5" width="17.109375" customWidth="1"/>
-    <col min="10" max="10" width="38.21875" customWidth="1"/>
-    <col min="11" max="11" width="20.5546875" customWidth="1"/>
-    <col min="13" max="13" width="20.5546875" customWidth="1"/>
-    <col min="15" max="15" width="20.21875" customWidth="1"/>
+    <col min="4" max="4" width="17.5703125" customWidth="1"/>
+    <col min="5" max="5" width="17.140625" customWidth="1"/>
+    <col min="10" max="10" width="38.28515625" customWidth="1"/>
+    <col min="11" max="11" width="20.5703125" customWidth="1"/>
+    <col min="13" max="13" width="20.5703125" customWidth="1"/>
+    <col min="15" max="15" width="20.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="3:14" ht="93.6" x14ac:dyDescent="1.75">
+    <row r="1" spans="3:14" ht="93.75" x14ac:dyDescent="1.4">
       <c r="D1" s="6" t="s">
         <v>314</v>
       </c>
     </row>
-    <row r="3" spans="3:14" x14ac:dyDescent="0.3">
+    <row r="3" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C3">
         <v>1000000</v>
       </c>
     </row>
-    <row r="4" spans="3:14" x14ac:dyDescent="0.3">
+    <row r="4" spans="3:14" x14ac:dyDescent="0.25">
       <c r="L4" t="s">
         <v>307</v>
       </c>
@@ -9394,7 +9394,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="5" spans="3:14" x14ac:dyDescent="0.3">
+    <row r="5" spans="3:14" x14ac:dyDescent="0.25">
       <c r="L5">
         <v>65000</v>
       </c>
@@ -9402,7 +9402,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="3:14" x14ac:dyDescent="0.3">
+    <row r="7" spans="3:14" x14ac:dyDescent="0.25">
       <c r="D7" t="s">
         <v>305</v>
       </c>
@@ -9419,7 +9419,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="8" spans="3:14" x14ac:dyDescent="0.3">
+    <row r="8" spans="3:14" x14ac:dyDescent="0.25">
       <c r="D8">
         <v>8000</v>
       </c>
@@ -9440,13 +9440,13 @@
         <v>313</v>
       </c>
     </row>
-    <row r="9" spans="3:14" x14ac:dyDescent="0.3">
+    <row r="9" spans="3:14" x14ac:dyDescent="0.25">
       <c r="M9">
         <f>J14-ROUND(J14,0)</f>
         <v>0.24615384615384617</v>
       </c>
     </row>
-    <row r="12" spans="3:14" x14ac:dyDescent="0.3">
+    <row r="12" spans="3:14" x14ac:dyDescent="0.25">
       <c r="D12">
         <f>(E8*C3)/((F8+1)*(G8+1))</f>
         <v>39.99972500189061</v>
@@ -9455,7 +9455,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="13" spans="3:14" x14ac:dyDescent="0.3">
+    <row r="13" spans="3:14" x14ac:dyDescent="0.25">
       <c r="J13" t="s">
         <v>308</v>
       </c>
@@ -9464,19 +9464,19 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="14" spans="3:14" x14ac:dyDescent="0.3">
+    <row r="14" spans="3:14" x14ac:dyDescent="0.25">
       <c r="J14">
         <f>E8*C3/(D8*(L5))</f>
         <v>0.24615384615384617</v>
       </c>
     </row>
-    <row r="15" spans="3:14" x14ac:dyDescent="0.3">
+    <row r="15" spans="3:14" x14ac:dyDescent="0.25">
       <c r="J15">
         <f>TRUNC(J14)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="3:14" x14ac:dyDescent="0.3">
+    <row r="16" spans="3:14" x14ac:dyDescent="0.25">
       <c r="D16">
         <f>E8*C3/D8</f>
         <v>16000</v>
@@ -9485,7 +9485,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="17" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:16" x14ac:dyDescent="0.25">
       <c r="J17" t="s">
         <v>309</v>
       </c>
@@ -9493,7 +9493,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="18" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:16" x14ac:dyDescent="0.25">
       <c r="D18">
         <f>E8*C3/D16</f>
         <v>8000</v>
@@ -9507,7 +9507,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="23" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B23" s="5"/>
       <c r="C23" s="5"/>
       <c r="D23" s="5"/>
@@ -9523,7 +9523,7 @@
       <c r="N23" s="5"/>
       <c r="O23" s="5"/>
     </row>
-    <row r="28" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:16" x14ac:dyDescent="0.25">
       <c r="D28" t="s">
         <v>317</v>
       </c>
@@ -9531,7 +9531,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="29" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:16" x14ac:dyDescent="0.25">
       <c r="D29">
         <v>1000000</v>
       </c>
@@ -9543,7 +9543,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="30" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:16" x14ac:dyDescent="0.25">
       <c r="D30" t="s">
         <v>315</v>
       </c>
@@ -9579,7 +9579,7 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="31" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:16" x14ac:dyDescent="0.25">
       <c r="D31">
         <v>2000</v>
       </c>
@@ -9617,7 +9617,7 @@
         <v>0.59998942068653971</v>
       </c>
     </row>
-    <row r="32" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:16" x14ac:dyDescent="0.25">
       <c r="I32">
         <v>20</v>
       </c>
@@ -9642,7 +9642,7 @@
         <v>19.999645006301137</v>
       </c>
     </row>
-    <row r="33" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="33" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I33">
         <f>50+I32</f>
         <v>70</v>
@@ -9668,7 +9668,7 @@
         <v>69.998744397522373</v>
       </c>
     </row>
-    <row r="34" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="34" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I34">
         <f t="shared" ref="I34:I97" si="5">50+I33</f>
         <v>120</v>
@@ -9694,7 +9694,7 @@
         <v>119.9978400388793</v>
       </c>
     </row>
-    <row r="35" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="35" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I35">
         <f t="shared" si="5"/>
         <v>170</v>
@@ -9724,7 +9724,7 @@
         <v>169.99692943046216</v>
       </c>
     </row>
-    <row r="36" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="36" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I36">
         <f t="shared" si="5"/>
         <v>220</v>
@@ -9754,7 +9754,7 @@
         <v>219.99606757029218</v>
       </c>
     </row>
-    <row r="37" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="37" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I37">
         <f t="shared" si="5"/>
         <v>270</v>
@@ -9784,7 +9784,7 @@
         <v>269.99498821803121</v>
       </c>
     </row>
-    <row r="38" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="38" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I38">
         <f t="shared" si="5"/>
         <v>320</v>
@@ -9814,7 +9814,7 @@
         <v>319.99424010367812</v>
       </c>
     </row>
-    <row r="39" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="39" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I39">
         <f t="shared" si="5"/>
         <v>370</v>
@@ -9844,7 +9844,7 @@
         <v>369.99315512663014</v>
       </c>
     </row>
-    <row r="40" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="40" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I40">
         <f t="shared" si="5"/>
         <v>420</v>
@@ -9874,7 +9874,7 @@
         <v>419.99228264180647</v>
       </c>
     </row>
-    <row r="41" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="41" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I41">
         <f t="shared" si="5"/>
         <v>470</v>
@@ -9904,7 +9904,7 @@
         <v>469.99033582371959</v>
       </c>
     </row>
-    <row r="42" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="42" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I42">
         <f t="shared" si="5"/>
         <v>520</v>
@@ -9934,7 +9934,7 @@
         <v>519.9898601977261</v>
       </c>
     </row>
-    <row r="43" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="43" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I43">
         <f t="shared" si="5"/>
         <v>570</v>
@@ -9964,7 +9964,7 @@
         <v>569.98984705584928</v>
       </c>
     </row>
-    <row r="44" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="44" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I44">
         <f t="shared" si="5"/>
         <v>620</v>
@@ -9994,7 +9994,7 @@
         <v>619.98798773273768</v>
       </c>
     </row>
-    <row r="45" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="45" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I45">
         <f t="shared" si="5"/>
         <v>670</v>
@@ -10024,7 +10024,7 @@
         <v>669.98597216870769</v>
       </c>
     </row>
-    <row r="46" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="46" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I46">
         <f t="shared" si="5"/>
         <v>720</v>
@@ -10054,7 +10054,7 @@
         <v>719.98704023327582</v>
       </c>
     </row>
-    <row r="47" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="47" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I47">
         <f t="shared" si="5"/>
         <v>770</v>
@@ -10084,7 +10084,7 @@
         <v>769.98517778532755</v>
       </c>
     </row>
-    <row r="48" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="48" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I48">
         <f t="shared" si="5"/>
         <v>820</v>
@@ -10114,7 +10114,7 @@
         <v>819.98319034459792</v>
       </c>
     </row>
-    <row r="49" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="49" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I49">
         <f t="shared" si="5"/>
         <v>870</v>
@@ -10144,7 +10144,7 @@
         <v>869.98107791155542</v>
       </c>
     </row>
-    <row r="50" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="50" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I50">
         <f t="shared" si="5"/>
         <v>920</v>
@@ -10174,7 +10174,7 @@
         <v>919.97884048666879</v>
       </c>
     </row>
-    <row r="51" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="51" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I51">
         <f t="shared" si="5"/>
         <v>970</v>
@@ -10204,7 +10204,7 @@
         <v>969.98235844585577</v>
       </c>
     </row>
-    <row r="52" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="52" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I52">
         <f t="shared" si="5"/>
         <v>1020</v>
@@ -10234,7 +10234,7 @@
         <v>1019.9804928730738</v>
       </c>
     </row>
-    <row r="53" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="53" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I53">
         <f t="shared" si="5"/>
         <v>1070</v>
@@ -10264,7 +10264,7 @@
         <v>1069.9785335556708</v>
       </c>
     </row>
-    <row r="54" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="54" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I54">
         <f t="shared" si="5"/>
         <v>1120</v>
@@ -10294,7 +10294,7 @@
         <v>1119.9764804939098</v>
       </c>
     </row>
-    <row r="55" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="55" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I55">
         <f t="shared" si="5"/>
         <v>1170</v>
@@ -10324,7 +10324,7 @@
         <v>1169.9743336880547</v>
       </c>
     </row>
-    <row r="56" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="56" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I56">
         <f t="shared" si="5"/>
         <v>1220</v>
@@ -10354,7 +10354,7 @@
         <v>1219.9720931383697</v>
       </c>
     </row>
-    <row r="57" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="57" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I57">
         <f t="shared" si="5"/>
         <v>1270</v>
@@ -10384,7 +10384,7 @@
         <v>1269.9697588451177</v>
       </c>
     </row>
-    <row r="58" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="58" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I58">
         <f t="shared" si="5"/>
         <v>1320</v>
@@ -10414,7 +10414,7 @@
         <v>1319.9673308085623</v>
       </c>
     </row>
-    <row r="59" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="59" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I59">
         <f t="shared" si="5"/>
         <v>1370</v>
@@ -10444,7 +10444,7 @@
         <v>1369.9648090289681</v>
       </c>
     </row>
-    <row r="60" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="60" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I60">
         <f t="shared" si="5"/>
         <v>1420</v>
@@ -10474,7 +10474,7 @@
         <v>1419.9747954473808</v>
       </c>
     </row>
-    <row r="61" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="61" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I61">
         <f t="shared" si="5"/>
         <v>1470</v>
@@ -10504,7 +10504,7 @@
         <v>1469.9729892463226</v>
       </c>
     </row>
-    <row r="62" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="62" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I62">
         <f t="shared" si="5"/>
         <v>1520</v>
@@ -10534,7 +10534,7 @@
         <v>1519.9711205487097</v>
       </c>
     </row>
-    <row r="63" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="63" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I63">
         <f t="shared" si="5"/>
         <v>1570</v>
@@ -10564,7 +10564,7 @@
         <v>1569.969189354659</v>
       </c>
     </row>
-    <row r="64" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="64" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I64">
         <f t="shared" si="5"/>
         <v>1620</v>
@@ -10594,7 +10594,7 @@
         <v>1619.9671956642878</v>
       </c>
     </row>
-    <row r="65" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="65" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I65">
         <f t="shared" si="5"/>
         <v>1670</v>
@@ -10624,7 +10624,7 @@
         <v>1669.9651394777134</v>
       </c>
     </row>
-    <row r="66" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="66" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I66">
         <f t="shared" si="5"/>
         <v>1720</v>
@@ -10654,7 +10654,7 @@
         <v>1719.9630207950531</v>
       </c>
     </row>
-    <row r="67" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="67" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I67">
         <f t="shared" si="5"/>
         <v>1770</v>
@@ -10684,7 +10684,7 @@
         <v>1769.9608396164233</v>
       </c>
     </row>
-    <row r="68" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="68" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I68">
         <f t="shared" si="5"/>
         <v>1820</v>
@@ -10714,7 +10714,7 @@
         <v>1819.9585959419423</v>
       </c>
     </row>
-    <row r="69" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="69" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I69">
         <f t="shared" si="5"/>
         <v>1870</v>
@@ -10744,7 +10744,7 @@
         <v>1869.9562897717265</v>
       </c>
     </row>
-    <row r="70" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="70" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I70">
         <f t="shared" si="5"/>
         <v>1920</v>
@@ -10774,7 +10774,7 @@
         <v>1919.9539211058936</v>
       </c>
     </row>
-    <row r="71" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="71" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I71">
         <f t="shared" si="5"/>
         <v>1970</v>
@@ -10804,7 +10804,7 @@
         <v>1969.9514899445601</v>
       </c>
     </row>
-    <row r="72" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="72" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I72">
         <f t="shared" si="5"/>
         <v>2020</v>
@@ -10834,7 +10834,7 @@
         <v>2019.9489962878436</v>
       </c>
     </row>
-    <row r="73" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="73" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I73">
         <f t="shared" si="5"/>
         <v>2070</v>
@@ -10864,7 +10864,7 @@
         <v>2069.9464401358614</v>
       </c>
     </row>
-    <row r="74" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="74" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I74">
         <f t="shared" si="5"/>
         <v>2120</v>
@@ -10894,7 +10894,7 @@
         <v>2119.9438214887305</v>
       </c>
     </row>
-    <row r="75" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="75" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I75">
         <f t="shared" si="5"/>
         <v>2170</v>
@@ -10924,7 +10924,7 @@
         <v>2169.9411403465683</v>
       </c>
     </row>
-    <row r="76" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="76" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I76">
         <f t="shared" si="5"/>
         <v>2220</v>
@@ -10954,7 +10954,7 @@
         <v>2219.9383967094914</v>
       </c>
     </row>
-    <row r="77" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="77" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I77">
         <f t="shared" si="5"/>
         <v>2270</v>
@@ -10984,7 +10984,7 @@
         <v>2269.9355905776174</v>
       </c>
     </row>
-    <row r="78" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="78" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I78">
         <f t="shared" si="5"/>
         <v>2320</v>
@@ -11014,7 +11014,7 @@
         <v>2319.9327219510637</v>
       </c>
     </row>
-    <row r="79" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="79" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I79">
         <f t="shared" si="5"/>
         <v>2370</v>
@@ -11044,7 +11044,7 @@
         <v>2369.9297908299468</v>
       </c>
     </row>
-    <row r="80" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="80" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I80">
         <f t="shared" si="5"/>
         <v>2420</v>
@@ -11074,7 +11074,7 @@
         <v>2419.9267972143844</v>
       </c>
     </row>
-    <row r="81" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="81" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I81">
         <f t="shared" si="5"/>
         <v>2470</v>
@@ -11104,7 +11104,7 @@
         <v>2469.9237411044933</v>
       </c>
     </row>
-    <row r="82" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="82" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I82">
         <f t="shared" si="5"/>
         <v>2520</v>
@@ -11134,7 +11134,7 @@
         <v>2519.9206225003913</v>
       </c>
     </row>
-    <row r="83" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="83" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I83">
         <f t="shared" si="5"/>
         <v>2570</v>
@@ -11164,7 +11164,7 @@
         <v>2569.917441402195</v>
       </c>
     </row>
-    <row r="84" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="84" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I84">
         <f t="shared" si="5"/>
         <v>2620</v>
@@ -11194,7 +11194,7 @@
         <v>2619.914197810022</v>
       </c>
     </row>
-    <row r="85" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="85" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I85">
         <f t="shared" si="5"/>
         <v>2670</v>
@@ -11224,7 +11224,7 @@
         <v>2669.9108917239887</v>
       </c>
     </row>
-    <row r="86" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="86" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I86">
         <f t="shared" si="5"/>
         <v>2720</v>
@@ -11254,7 +11254,7 @@
         <v>2719.907523144213</v>
       </c>
     </row>
-    <row r="87" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="87" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I87">
         <f t="shared" si="5"/>
         <v>2770</v>
@@ -11284,7 +11284,7 @@
         <v>2769.9040920708121</v>
       </c>
     </row>
-    <row r="88" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="88" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I88">
         <f t="shared" si="5"/>
         <v>2820</v>
@@ -11314,7 +11314,7 @@
         <v>2819.9005985039025</v>
       </c>
     </row>
-    <row r="89" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="89" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I89">
         <f t="shared" si="5"/>
         <v>2870</v>
@@ -11344,7 +11344,7 @@
         <v>2869.9485202984174</v>
       </c>
     </row>
-    <row r="90" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="90" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I90">
         <f t="shared" si="5"/>
         <v>2920</v>
@@ -11374,7 +11374,7 @@
         <v>2919.9467109725247</v>
       </c>
     </row>
-    <row r="91" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="91" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I91">
         <f t="shared" si="5"/>
         <v>2970</v>
@@ -11404,7 +11404,7 @@
         <v>2969.944870398343</v>
       </c>
     </row>
-    <row r="92" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="92" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I92">
         <f t="shared" si="5"/>
         <v>3020</v>
@@ -11434,7 +11434,7 @@
         <v>3019.942998575902</v>
       </c>
     </row>
-    <row r="93" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="93" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I93">
         <f t="shared" si="5"/>
         <v>3070</v>
@@ -11464,7 +11464,7 @@
         <v>3069.9410955052299</v>
       </c>
     </row>
-    <row r="94" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="94" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I94">
         <f t="shared" si="5"/>
         <v>3120</v>
@@ -11494,7 +11494,7 @@
         <v>3119.9391611863571</v>
       </c>
     </row>
-    <row r="95" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="95" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I95">
         <f t="shared" si="5"/>
         <v>3170</v>
@@ -11524,7 +11524,7 @@
         <v>3169.9371956193118</v>
       </c>
     </row>
-    <row r="96" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="96" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I96">
         <f t="shared" si="5"/>
         <v>3220</v>
@@ -11554,7 +11554,7 @@
         <v>3219.935198804124</v>
       </c>
     </row>
-    <row r="97" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="97" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I97">
         <f t="shared" si="5"/>
         <v>3270</v>
@@ -11584,7 +11584,7 @@
         <v>3269.9331707408232</v>
       </c>
     </row>
-    <row r="98" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="98" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I98">
         <f t="shared" ref="I98:I161" si="13">50+I97</f>
         <v>3320</v>
@@ -11614,7 +11614,7 @@
         <v>3319.9311114294378</v>
       </c>
     </row>
-    <row r="99" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="99" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I99">
         <f t="shared" si="13"/>
         <v>3370</v>
@@ -11644,7 +11644,7 @@
         <v>3369.9290208699977</v>
       </c>
     </row>
-    <row r="100" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="100" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I100">
         <f t="shared" si="13"/>
         <v>3420</v>
@@ -11674,7 +11674,7 @@
         <v>3419.9268990625328</v>
       </c>
     </row>
-    <row r="101" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="101" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I101">
         <f t="shared" si="13"/>
         <v>3470</v>
@@ -11704,7 +11704,7 @@
         <v>3469.924746007071</v>
       </c>
     </row>
-    <row r="102" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="102" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I102">
         <f t="shared" si="13"/>
         <v>3520</v>
@@ -11734,7 +11734,7 @@
         <v>3519.9225617036423</v>
       </c>
     </row>
-    <row r="103" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="103" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I103">
         <f t="shared" si="13"/>
         <v>3570</v>
@@ -11764,7 +11764,7 @@
         <v>3569.9203461522766</v>
       </c>
     </row>
-    <row r="104" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="104" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I104">
         <f t="shared" si="13"/>
         <v>3620</v>
@@ -11794,7 +11794,7 @@
         <v>3619.9180993530017</v>
       </c>
     </row>
-    <row r="105" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="105" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I105">
         <f t="shared" si="13"/>
         <v>3670</v>
@@ -11824,7 +11824,7 @@
         <v>3669.915821305849</v>
       </c>
     </row>
-    <row r="106" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="106" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I106">
         <f t="shared" si="13"/>
         <v>3720</v>
@@ -11854,7 +11854,7 @@
         <v>3719.9135120108458</v>
       </c>
     </row>
-    <row r="107" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="107" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I107">
         <f t="shared" si="13"/>
         <v>3770</v>
@@ -11884,7 +11884,7 @@
         <v>3769.9111714680221</v>
       </c>
     </row>
-    <row r="108" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="108" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I108">
         <f t="shared" si="13"/>
         <v>3820</v>
@@ -11914,7 +11914,7 @@
         <v>3819.9087996774078</v>
       </c>
     </row>
-    <row r="109" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="109" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I109">
         <f t="shared" si="13"/>
         <v>3870</v>
@@ -11944,7 +11944,7 @@
         <v>3869.9063966390313</v>
       </c>
     </row>
-    <row r="110" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="110" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I110">
         <f t="shared" si="13"/>
         <v>3920</v>
@@ -11974,7 +11974,7 @@
         <v>3919.903962352922</v>
       </c>
     </row>
-    <row r="111" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="111" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I111">
         <f t="shared" si="13"/>
         <v>3970</v>
@@ -12004,7 +12004,7 @@
         <v>3969.90149681911</v>
       </c>
     </row>
-    <row r="112" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="112" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I112">
         <f t="shared" si="13"/>
         <v>4020</v>
@@ -12034,7 +12034,7 @@
         <v>4019.8990000376243</v>
       </c>
     </row>
-    <row r="113" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="113" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I113">
         <f t="shared" si="13"/>
         <v>4070</v>
@@ -12064,7 +12064,7 @@
         <v>4069.8964720084932</v>
       </c>
     </row>
-    <row r="114" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="114" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I114">
         <f t="shared" si="13"/>
         <v>4120</v>
@@ -12094,7 +12094,7 @@
         <v>4119.8939127317472</v>
       </c>
     </row>
-    <row r="115" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="115" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I115">
         <f t="shared" si="13"/>
         <v>4170</v>
@@ -12124,7 +12124,7 @@
         <v>4169.8913222074152</v>
       </c>
     </row>
-    <row r="116" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="116" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I116">
         <f t="shared" si="13"/>
         <v>4220</v>
@@ -12154,7 +12154,7 @@
         <v>4219.8887004355265</v>
       </c>
     </row>
-    <row r="117" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="117" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I117">
         <f t="shared" si="13"/>
         <v>4270</v>
@@ -12184,7 +12184,7 @@
         <v>4269.8860474161092</v>
       </c>
     </row>
-    <row r="118" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="118" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I118">
         <f t="shared" si="13"/>
         <v>4320</v>
@@ -12214,7 +12214,7 @@
         <v>4319.8833631491952</v>
       </c>
     </row>
-    <row r="119" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="119" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I119">
         <f t="shared" si="13"/>
         <v>4370</v>
@@ -12244,7 +12244,7 @@
         <v>4369.8806476348118</v>
       </c>
     </row>
-    <row r="120" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="120" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I120">
         <f t="shared" si="13"/>
         <v>4420</v>
@@ -12274,7 +12274,7 @@
         <v>4419.8779008729889</v>
       </c>
     </row>
-    <row r="121" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="121" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I121">
         <f t="shared" si="13"/>
         <v>4470</v>
@@ -12304,7 +12304,7 @@
         <v>4469.8751228637548</v>
       </c>
     </row>
-    <row r="122" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="122" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I122">
         <f t="shared" si="13"/>
         <v>4520</v>
@@ -12334,7 +12334,7 @@
         <v>4519.8723136071403</v>
       </c>
     </row>
-    <row r="123" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="123" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I123">
         <f t="shared" si="13"/>
         <v>4570</v>
@@ -12364,7 +12364,7 @@
         <v>4569.8694731031737</v>
       </c>
     </row>
-    <row r="124" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="124" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I124">
         <f t="shared" si="13"/>
         <v>4620</v>
@@ -12394,7 +12394,7 @@
         <v>4619.8666013518859</v>
       </c>
     </row>
-    <row r="125" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="125" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I125">
         <f t="shared" si="13"/>
         <v>4670</v>
@@ -12424,7 +12424,7 @@
         <v>4669.8636983533042</v>
       </c>
     </row>
-    <row r="126" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="126" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I126">
         <f t="shared" si="13"/>
         <v>4720</v>
@@ -12454,7 +12454,7 @@
         <v>4719.8607641074586</v>
       </c>
     </row>
-    <row r="127" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="127" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I127">
         <f t="shared" si="13"/>
         <v>4770</v>
@@ -12484,7 +12484,7 @@
         <v>4769.8577986143782</v>
       </c>
     </row>
-    <row r="128" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="128" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I128">
         <f t="shared" si="13"/>
         <v>4820</v>
@@ -12514,7 +12514,7 @@
         <v>4819.8548018740939</v>
       </c>
     </row>
-    <row r="129" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="129" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I129">
         <f t="shared" si="13"/>
         <v>4870</v>
@@ -12544,7 +12544,7 @@
         <v>4869.8517738866331</v>
       </c>
     </row>
-    <row r="130" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="130" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I130">
         <f t="shared" si="13"/>
         <v>4920</v>
@@ -12574,7 +12574,7 @@
         <v>4919.8487146520247</v>
       </c>
     </row>
-    <row r="131" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="131" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I131">
         <f t="shared" si="13"/>
         <v>4970</v>
@@ -12604,7 +12604,7 @@
         <v>4969.8456241702988</v>
       </c>
     </row>
-    <row r="132" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="132" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I132">
         <f t="shared" si="13"/>
         <v>5020</v>
@@ -12634,7 +12634,7 @@
         <v>5019.8425024414864</v>
       </c>
     </row>
-    <row r="133" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="133" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I133">
         <f t="shared" si="13"/>
         <v>5070</v>
@@ -12664,7 +12664,7 @@
         <v>5069.8393494656139</v>
       </c>
     </row>
-    <row r="134" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="134" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I134">
         <f t="shared" si="13"/>
         <v>5120</v>
@@ -12694,7 +12694,7 @@
         <v>5119.836165242712</v>
       </c>
     </row>
-    <row r="135" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="135" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I135">
         <f t="shared" si="13"/>
         <v>5170</v>
@@ -12724,7 +12724,7 @@
         <v>5169.8329497728109</v>
       </c>
     </row>
-    <row r="136" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="136" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I136">
         <f t="shared" si="13"/>
         <v>5220</v>
@@ -12754,7 +12754,7 @@
         <v>5219.8297030559379</v>
       </c>
     </row>
-    <row r="137" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="137" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I137">
         <f t="shared" si="13"/>
         <v>5270</v>
@@ -12784,7 +12784,7 @@
         <v>5269.8264250921238</v>
       </c>
     </row>
-    <row r="138" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="138" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I138">
         <f t="shared" si="13"/>
         <v>5320</v>
@@ -12814,7 +12814,7 @@
         <v>5319.8231158813969</v>
       </c>
     </row>
-    <row r="139" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="139" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I139">
         <f t="shared" si="13"/>
         <v>5370</v>
@@ -12844,7 +12844,7 @@
         <v>5369.8197754237872</v>
       </c>
     </row>
-    <row r="140" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="140" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I140">
         <f t="shared" si="13"/>
         <v>5420</v>
@@ -12874,7 +12874,7 @@
         <v>5419.8164037193237</v>
       </c>
     </row>
-    <row r="141" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="141" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I141">
         <f t="shared" si="13"/>
         <v>5470</v>
@@ -12904,7 +12904,7 @@
         <v>5469.8130007680365</v>
       </c>
     </row>
-    <row r="142" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="142" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I142">
         <f t="shared" si="13"/>
         <v>5520</v>
@@ -12934,7 +12934,7 @@
         <v>5519.8095665699529</v>
       </c>
     </row>
-    <row r="143" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="143" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I143">
         <f t="shared" si="13"/>
         <v>5570</v>
@@ -12964,7 +12964,7 @@
         <v>5569.8061011251048</v>
       </c>
     </row>
-    <row r="144" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="144" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I144">
         <f t="shared" si="13"/>
         <v>5620</v>
@@ -12994,7 +12994,7 @@
         <v>5619.8026044335193</v>
       </c>
     </row>
-    <row r="145" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="145" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I145">
         <f t="shared" si="13"/>
         <v>5670</v>
@@ -13024,7 +13024,7 @@
         <v>5669.7990764952274</v>
       </c>
     </row>
-    <row r="146" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="146" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I146">
         <f t="shared" si="13"/>
         <v>5720</v>
@@ -13054,7 +13054,7 @@
         <v>5719.7955173102564</v>
       </c>
     </row>
-    <row r="147" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="147" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I147">
         <f t="shared" si="13"/>
         <v>5770</v>
@@ -13084,7 +13084,7 @@
         <v>5769.7919268786372</v>
       </c>
     </row>
-    <row r="148" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="148" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I148">
         <f t="shared" si="13"/>
         <v>5820</v>
@@ -13114,7 +13114,7 @@
         <v>5819.788305200399</v>
       </c>
     </row>
-    <row r="149" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="149" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I149">
         <f t="shared" si="13"/>
         <v>5870</v>
@@ -13144,7 +13144,7 @@
         <v>5869.7846522755699</v>
       </c>
     </row>
-    <row r="150" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="150" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I150">
         <f t="shared" si="13"/>
         <v>5920</v>
@@ -13174,7 +13174,7 @@
         <v>5919.7809681041799</v>
       </c>
     </row>
-    <row r="151" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="151" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I151">
         <f t="shared" si="13"/>
         <v>5970</v>
@@ -13204,7 +13204,7 @@
         <v>5969.7772526862591</v>
       </c>
     </row>
-    <row r="152" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="152" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I152">
         <f t="shared" si="13"/>
         <v>6020</v>
@@ -13234,7 +13234,7 @@
         <v>6019.7735060218356</v>
       </c>
     </row>
-    <row r="153" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="153" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I153">
         <f t="shared" si="13"/>
         <v>6070</v>
@@ -13264,7 +13264,7 @@
         <v>6069.7697281109404</v>
       </c>
     </row>
-    <row r="154" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="154" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I154">
         <f t="shared" si="13"/>
         <v>6120</v>
@@ -13294,7 +13294,7 @@
         <v>6119.7659189536007</v>
       </c>
     </row>
-    <row r="155" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="155" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I155">
         <f t="shared" si="13"/>
         <v>6170</v>
@@ -13324,7 +13324,7 @@
         <v>6169.7620785498466</v>
       </c>
     </row>
-    <row r="156" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="156" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I156">
         <f t="shared" si="13"/>
         <v>6220</v>
@@ -13354,7 +13354,7 @@
         <v>6219.7582068997071</v>
       </c>
     </row>
-    <row r="157" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="157" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I157">
         <f t="shared" si="13"/>
         <v>6270</v>
@@ -13384,7 +13384,7 @@
         <v>6269.7543040032115</v>
       </c>
     </row>
-    <row r="158" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="158" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I158">
         <f t="shared" si="13"/>
         <v>6320</v>
@@ -13414,7 +13414,7 @@
         <v>6319.7503698603905</v>
       </c>
     </row>
-    <row r="159" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="159" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I159">
         <f t="shared" si="13"/>
         <v>6370</v>
@@ -13444,7 +13444,7 @@
         <v>6369.7464044712724</v>
       </c>
     </row>
-    <row r="160" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="160" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I160">
         <f t="shared" si="13"/>
         <v>6420</v>
@@ -13474,7 +13474,7 @@
         <v>6419.7424078358863</v>
       </c>
     </row>
-    <row r="161" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="161" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I161">
         <f t="shared" si="13"/>
         <v>6470</v>
@@ -13504,7 +13504,7 @@
         <v>6469.7383799542604</v>
       </c>
     </row>
-    <row r="162" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="162" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I162">
         <f t="shared" ref="I162:I225" si="20">50+I161</f>
         <v>6520</v>
@@ -13534,7 +13534,7 @@
         <v>6519.7343208264265</v>
       </c>
     </row>
-    <row r="163" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="163" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I163">
         <f t="shared" si="20"/>
         <v>6570</v>
@@ -13564,7 +13564,7 @@
         <v>6569.7302304524128</v>
       </c>
     </row>
-    <row r="164" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="164" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I164">
         <f t="shared" si="20"/>
         <v>6620</v>
@@ -13594,7 +13594,7 @@
         <v>6619.7261088322475</v>
       </c>
     </row>
-    <row r="165" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="165" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I165">
         <f t="shared" si="20"/>
         <v>6670</v>
@@ -13624,7 +13624,7 @@
         <v>6669.7219559659607</v>
       </c>
     </row>
-    <row r="166" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="166" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I166">
         <f t="shared" si="20"/>
         <v>6720</v>
@@ -13654,7 +13654,7 @@
         <v>6719.7177718535822</v>
       </c>
     </row>
-    <row r="167" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="167" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I167">
         <f t="shared" si="20"/>
         <v>6770</v>
@@ -13684,7 +13684,7 @@
         <v>6769.7135564951404</v>
       </c>
     </row>
-    <row r="168" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="168" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I168">
         <f t="shared" si="20"/>
         <v>6820</v>
@@ -13714,7 +13714,7 @@
         <v>6819.7093098906662</v>
       </c>
     </row>
-    <row r="169" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="169" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I169">
         <f t="shared" si="20"/>
         <v>6870</v>
@@ -13744,7 +13744,7 @@
         <v>6869.7050320401868</v>
       </c>
     </row>
-    <row r="170" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="170" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I170">
         <f t="shared" si="20"/>
         <v>6920</v>
@@ -13774,7 +13774,7 @@
         <v>6919.7007229437331</v>
       </c>
     </row>
-    <row r="171" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="171" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I171">
         <f t="shared" si="20"/>
         <v>6970</v>
@@ -13804,7 +13804,7 @@
         <v>6969.6963826013325</v>
       </c>
     </row>
-    <row r="172" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="172" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I172">
         <f t="shared" si="20"/>
         <v>7020</v>
@@ -13834,7 +13834,7 @@
         <v>7019.6920110130168</v>
       </c>
     </row>
-    <row r="173" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="173" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I173">
         <f t="shared" si="20"/>
         <v>7070</v>
@@ -13864,7 +13864,7 @@
         <v>7069.6876081788141</v>
       </c>
     </row>
-    <row r="174" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="174" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I174">
         <f t="shared" si="20"/>
         <v>7120</v>
@@ -13894,7 +13894,7 @@
         <v>7119.6831740987527</v>
       </c>
     </row>
-    <row r="175" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="175" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I175">
         <f t="shared" si="20"/>
         <v>7170</v>
@@ -13924,7 +13924,7 @@
         <v>7169.6787087728635</v>
       </c>
     </row>
-    <row r="176" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="176" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I176">
         <f t="shared" si="20"/>
         <v>7220</v>
@@ -13954,7 +13954,7 @@
         <v>7219.6742122011738</v>
       </c>
     </row>
-    <row r="177" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="177" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I177">
         <f t="shared" si="20"/>
         <v>7270</v>
@@ -13984,7 +13984,7 @@
         <v>7269.6696843837153</v>
       </c>
     </row>
-    <row r="178" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="178" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I178">
         <f t="shared" si="20"/>
         <v>7320</v>
@@ -14014,7 +14014,7 @@
         <v>7319.6651253205173</v>
       </c>
     </row>
-    <row r="179" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="179" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I179">
         <f t="shared" si="20"/>
         <v>7370</v>
@@ -14044,7 +14044,7 @@
         <v>7369.6605350116051</v>
       </c>
     </row>
-    <row r="180" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="180" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I180">
         <f t="shared" si="20"/>
         <v>7420</v>
@@ -14074,7 +14074,7 @@
         <v>7419.6559134570134</v>
       </c>
     </row>
-    <row r="181" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="181" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I181">
         <f t="shared" si="20"/>
         <v>7470</v>
@@ -14104,7 +14104,7 @@
         <v>7469.6512606567685</v>
       </c>
     </row>
-    <row r="182" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="182" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I182">
         <f t="shared" si="20"/>
         <v>7520</v>
@@ -14134,7 +14134,7 @@
         <v>7519.6465766108995</v>
       </c>
     </row>
-    <row r="183" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="183" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I183">
         <f t="shared" si="20"/>
         <v>7570</v>
@@ -14164,7 +14164,7 @@
         <v>7569.6418613194364</v>
       </c>
     </row>
-    <row r="184" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="184" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I184">
         <f t="shared" si="20"/>
         <v>7620</v>
@@ -14194,7 +14194,7 @@
         <v>7619.6371147824093</v>
       </c>
     </row>
-    <row r="185" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="185" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I185">
         <f t="shared" si="20"/>
         <v>7670</v>
@@ -14224,7 +14224,7 @@
         <v>7669.6323369998454</v>
       </c>
     </row>
-    <row r="186" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="186" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I186">
         <f t="shared" si="20"/>
         <v>7720</v>
@@ -14254,7 +14254,7 @@
         <v>7719.6275279717756</v>
       </c>
     </row>
-    <row r="187" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="187" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I187">
         <f t="shared" si="20"/>
         <v>7770</v>
@@ -14284,7 +14284,7 @@
         <v>7769.6226876982291</v>
       </c>
     </row>
-    <row r="188" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="188" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I188">
         <f t="shared" si="20"/>
         <v>7820</v>
@@ -14314,7 +14314,7 @@
         <v>7819.6178161792341</v>
       </c>
     </row>
-    <row r="189" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="189" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I189">
         <f t="shared" si="20"/>
         <v>7870</v>
@@ -14344,7 +14344,7 @@
         <v>7869.6129134148214</v>
       </c>
     </row>
-    <row r="190" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="190" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I190">
         <f t="shared" si="20"/>
         <v>7920</v>
@@ -14374,7 +14374,7 @@
         <v>7919.6079794050193</v>
       </c>
     </row>
-    <row r="191" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="191" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I191">
         <f t="shared" si="20"/>
         <v>7970</v>
@@ -14404,7 +14404,7 @@
         <v>7969.6030141498577</v>
       </c>
     </row>
-    <row r="192" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="192" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I192">
         <f t="shared" si="20"/>
         <v>8020</v>
@@ -14434,7 +14434,7 @@
         <v>8019.5980176493649</v>
       </c>
     </row>
-    <row r="193" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="193" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I193">
         <f t="shared" si="20"/>
         <v>8070</v>
@@ -14464,7 +14464,7 @@
         <v>8069.5929899035727</v>
       </c>
     </row>
-    <row r="194" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="194" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I194">
         <f t="shared" si="20"/>
         <v>8120</v>
@@ -14494,7 +14494,7 @@
         <v>8119.5879309125066</v>
       </c>
     </row>
-    <row r="195" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="195" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I195">
         <f t="shared" si="20"/>
         <v>8170</v>
@@ -14524,7 +14524,7 @@
         <v>8169.5828406761975</v>
       </c>
     </row>
-    <row r="196" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="196" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I196">
         <f t="shared" si="20"/>
         <v>8220</v>
@@ -14554,7 +14554,7 @@
         <v>8219.5777191946763</v>
       </c>
     </row>
-    <row r="197" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="197" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I197">
         <f t="shared" si="20"/>
         <v>8270</v>
@@ -14584,7 +14584,7 @@
         <v>8269.5725664679703</v>
       </c>
     </row>
-    <row r="198" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="198" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I198">
         <f t="shared" si="20"/>
         <v>8320</v>
@@ -14614,7 +14614,7 @@
         <v>8319.5673824961104</v>
       </c>
     </row>
-    <row r="199" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="199" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I199">
         <f t="shared" si="20"/>
         <v>8370</v>
@@ -14644,7 +14644,7 @@
         <v>8369.562167279124</v>
       </c>
     </row>
-    <row r="200" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="200" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I200">
         <f t="shared" si="20"/>
         <v>8420</v>
@@ -14674,7 +14674,7 @@
         <v>8419.5569208170418</v>
       </c>
     </row>
-    <row r="201" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="201" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I201">
         <f t="shared" si="20"/>
         <v>8470</v>
@@ -14704,7 +14704,7 @@
         <v>8469.5516431098931</v>
       </c>
     </row>
-    <row r="202" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="202" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I202">
         <f t="shared" si="20"/>
         <v>8520</v>
@@ -14734,7 +14734,7 @@
         <v>8519.546334157707</v>
       </c>
     </row>
-    <row r="203" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="203" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I203">
         <f t="shared" si="20"/>
         <v>8570</v>
@@ -14764,7 +14764,7 @@
         <v>8569.5409939605106</v>
       </c>
     </row>
-    <row r="204" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="204" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I204">
         <f t="shared" si="20"/>
         <v>8620</v>
@@ -14794,7 +14794,7 @@
         <v>8619.5356225183368</v>
       </c>
     </row>
-    <row r="205" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="205" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I205">
         <f t="shared" si="20"/>
         <v>8670</v>
@@ -14824,7 +14824,7 @@
         <v>8669.5302198312129</v>
       </c>
     </row>
-    <row r="206" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="206" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I206">
         <f t="shared" si="20"/>
         <v>8720</v>
@@ -14854,7 +14854,7 @@
         <v>8719.5247858991697</v>
       </c>
     </row>
-    <row r="207" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="207" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I207">
         <f t="shared" si="20"/>
         <v>8770</v>
@@ -14884,7 +14884,7 @@
         <v>8769.5193207222328</v>
       </c>
     </row>
-    <row r="208" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="208" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I208">
         <f t="shared" si="20"/>
         <v>8820</v>
@@ -14914,7 +14914,7 @@
         <v>8819.5138243004349</v>
       </c>
     </row>
-    <row r="209" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="209" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I209">
         <f t="shared" si="20"/>
         <v>8870</v>
@@ -14944,7 +14944,7 @@
         <v>8869.508296633805</v>
       </c>
     </row>
-    <row r="210" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="210" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I210">
         <f t="shared" si="20"/>
         <v>8920</v>
@@ -14974,7 +14974,7 @@
         <v>8919.5027377223723</v>
       </c>
     </row>
-    <row r="211" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="211" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I211">
         <f t="shared" si="20"/>
         <v>8970</v>
@@ -15004,7 +15004,7 @@
         <v>8969.4971475661641</v>
       </c>
     </row>
-    <row r="212" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="212" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I212">
         <f t="shared" si="20"/>
         <v>9020</v>
@@ -15034,7 +15034,7 @@
         <v>9019.4915261652113</v>
       </c>
     </row>
-    <row r="213" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="213" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I213">
         <f t="shared" si="20"/>
         <v>9070</v>
@@ -15064,7 +15064,7 @@
         <v>9069.4858735195448</v>
       </c>
     </row>
-    <row r="214" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="214" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I214">
         <f t="shared" si="20"/>
         <v>9120</v>
@@ -15094,7 +15094,7 @@
         <v>9119.480189629192</v>
       </c>
     </row>
-    <row r="215" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="215" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I215">
         <f t="shared" si="20"/>
         <v>9170</v>
@@ -15124,7 +15124,7 @@
         <v>9169.47447449418</v>
       </c>
     </row>
-    <row r="216" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="216" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I216">
         <f t="shared" si="20"/>
         <v>9220</v>
@@ -15154,7 +15154,7 @@
         <v>9219.4687281145434</v>
       </c>
     </row>
-    <row r="217" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="217" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I217">
         <f t="shared" si="20"/>
         <v>9270</v>
@@ -15184,7 +15184,7 @@
         <v>9269.462950490306</v>
       </c>
     </row>
-    <row r="218" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="218" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I218">
         <f t="shared" si="20"/>
         <v>9320</v>
@@ -15214,7 +15214,7 @@
         <v>9319.4571416215003</v>
       </c>
     </row>
-    <row r="219" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="219" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I219">
         <f t="shared" si="20"/>
         <v>9370</v>
@@ -15244,7 +15244,7 @@
         <v>9369.4513015081538</v>
       </c>
     </row>
-    <row r="220" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="220" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I220">
         <f t="shared" si="20"/>
         <v>9420</v>
@@ -15274,7 +15274,7 @@
         <v>9419.4454301502992</v>
       </c>
     </row>
-    <row r="221" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="221" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I221">
         <f t="shared" si="20"/>
         <v>9470</v>
@@ -15304,7 +15304,7 @@
         <v>9469.4395275479637</v>
       </c>
     </row>
-    <row r="222" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="222" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I222">
         <f t="shared" si="20"/>
         <v>9520</v>
@@ -15334,7 +15334,7 @@
         <v>9519.4335937011747</v>
       </c>
     </row>
-    <row r="223" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="223" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I223">
         <f t="shared" si="20"/>
         <v>9570</v>
@@ -15364,7 +15364,7 @@
         <v>9569.4276286099648</v>
       </c>
     </row>
-    <row r="224" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="224" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I224">
         <f t="shared" si="20"/>
         <v>9620</v>
@@ -15394,7 +15394,7 @@
         <v>9619.4216322743596</v>
       </c>
     </row>
-    <row r="225" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="225" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I225">
         <f t="shared" si="20"/>
         <v>9670</v>
@@ -15424,7 +15424,7 @@
         <v>9669.4156046943899</v>
       </c>
     </row>
-    <row r="226" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="226" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I226">
         <f t="shared" ref="I226:I231" si="27">50+I225</f>
         <v>9720</v>
@@ -15454,7 +15454,7 @@
         <v>9719.4095458700867</v>
       </c>
     </row>
-    <row r="227" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="227" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I227">
         <f t="shared" si="27"/>
         <v>9770</v>
@@ -15484,7 +15484,7 @@
         <v>9769.403455801481</v>
       </c>
     </row>
-    <row r="228" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="228" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I228">
         <f t="shared" si="27"/>
         <v>9820</v>
@@ -15514,7 +15514,7 @@
         <v>9819.3973344885962</v>
       </c>
     </row>
-    <row r="229" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="229" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I229">
         <f t="shared" si="27"/>
         <v>9870</v>
@@ -15544,7 +15544,7 @@
         <v>9869.3911819314635</v>
       </c>
     </row>
-    <row r="230" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="230" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I230">
         <f t="shared" si="27"/>
         <v>9920</v>
@@ -15574,7 +15574,7 @@
         <v>9919.3849981301155</v>
       </c>
     </row>
-    <row r="231" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="231" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I231">
         <f t="shared" si="27"/>
         <v>9970</v>
@@ -15604,7 +15604,7 @@
         <v>9969.3787830845795</v>
       </c>
     </row>
-    <row r="232" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="232" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I232">
         <f>50+I231</f>
         <v>10020</v>
@@ -15634,7 +15634,7 @@
         <v>10019.372536794883</v>
       </c>
     </row>
-    <row r="233" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="233" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I233">
         <f t="shared" ref="I233:I254" si="29">50+I232</f>
         <v>10070</v>
@@ -15664,7 +15664,7 @@
         <v>10069.366259261058</v>
       </c>
     </row>
-    <row r="234" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="234" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I234">
         <f t="shared" si="29"/>
         <v>10120</v>
@@ -15694,7 +15694,7 @@
         <v>10119.359950483131</v>
       </c>
     </row>
-    <row r="235" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="235" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I235">
         <f t="shared" si="29"/>
         <v>10170</v>
@@ -15724,7 +15724,7 @@
         <v>10169.353610461136</v>
       </c>
     </row>
-    <row r="236" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="236" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I236">
         <f t="shared" si="29"/>
         <v>10220</v>
@@ -15754,7 +15754,7 @@
         <v>10219.347239195096</v>
       </c>
     </row>
-    <row r="237" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="237" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I237">
         <f t="shared" si="29"/>
         <v>10270</v>
@@ -15784,7 +15784,7 @@
         <v>10269.340836685045</v>
       </c>
     </row>
-    <row r="238" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="238" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I238">
         <f t="shared" si="29"/>
         <v>10320</v>
@@ -15814,7 +15814,7 @@
         <v>10319.33440293101</v>
       </c>
     </row>
-    <row r="239" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="239" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I239">
         <f t="shared" si="29"/>
         <v>10370</v>
@@ -15844,7 +15844,7 @@
         <v>10369.327937933023</v>
       </c>
     </row>
-    <row r="240" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="240" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I240">
         <f t="shared" si="29"/>
         <v>10420</v>
@@ -15874,7 +15874,7 @@
         <v>10419.321441691109</v>
       </c>
     </row>
-    <row r="241" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="241" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I241">
         <f t="shared" si="29"/>
         <v>10470</v>
@@ -15904,7 +15904,7 @@
         <v>10469.314914205301</v>
       </c>
     </row>
-    <row r="242" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="242" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I242">
         <f t="shared" si="29"/>
         <v>10520</v>
@@ -15934,7 +15934,7 @@
         <v>10519.308355475627</v>
       </c>
     </row>
-    <row r="243" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="243" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I243">
         <f t="shared" si="29"/>
         <v>10570</v>
@@ -15964,7 +15964,7 @@
         <v>10569.301765502116</v>
       </c>
     </row>
-    <row r="244" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="244" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I244">
         <f t="shared" si="29"/>
         <v>10620</v>
@@ -15994,7 +15994,7 @@
         <v>10619.295144284799</v>
       </c>
     </row>
-    <row r="245" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="245" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I245">
         <f t="shared" si="29"/>
         <v>10670</v>
@@ -16024,7 +16024,7 @@
         <v>10669.288491823701</v>
       </c>
     </row>
-    <row r="246" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="246" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I246">
         <f t="shared" si="29"/>
         <v>10720</v>
@@ -16054,7 +16054,7 @@
         <v>10719.281808118856</v>
       </c>
     </row>
-    <row r="247" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="247" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I247">
         <f t="shared" si="29"/>
         <v>10770</v>
@@ -16084,7 +16084,7 @@
         <v>10769.275093170292</v>
       </c>
     </row>
-    <row r="248" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="248" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I248">
         <f t="shared" si="29"/>
         <v>10820</v>
@@ -16114,7 +16114,7 @@
         <v>10819.268346978037</v>
       </c>
     </row>
-    <row r="249" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="249" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I249">
         <f t="shared" si="29"/>
         <v>10870</v>
@@ -16144,7 +16144,7 @@
         <v>10869.261569542119</v>
       </c>
     </row>
-    <row r="250" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="250" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I250">
         <f t="shared" si="29"/>
         <v>10920</v>
@@ -16174,7 +16174,7 @@
         <v>10919.254760862572</v>
       </c>
     </row>
-    <row r="251" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="251" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I251">
         <f t="shared" si="29"/>
         <v>10970</v>
@@ -16204,7 +16204,7 @@
         <v>10969.247920939421</v>
       </c>
     </row>
-    <row r="252" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="252" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I252">
         <f t="shared" si="29"/>
         <v>11020</v>
@@ -16234,7 +16234,7 @@
         <v>11019.241049772698</v>
       </c>
     </row>
-    <row r="253" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="253" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I253">
         <f t="shared" si="29"/>
         <v>11070</v>
@@ -16264,7 +16264,7 @@
         <v>11069.234147362429</v>
       </c>
     </row>
-    <row r="254" spans="9:15" x14ac:dyDescent="0.3">
+    <row r="254" spans="9:15" x14ac:dyDescent="0.25">
       <c r="I254">
         <f t="shared" si="29"/>
         <v>11120</v>

</xml_diff>